<commit_message>
Synchronize verified EEAI publication masters
</commit_message>
<xml_diff>
--- a/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
+++ b/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R540fa94d126e4844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="Ref3802402f1f41db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="Rb48d95a0360b4a68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="R0019d453500c4b4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,12 +32,17 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1F33"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -52,7 +57,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -136,6 +141,16 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -389,37 +404,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
-      <x:c r="A1" s="18" t="str">
+      <x:c r="A1" s="35" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="B1" s="18" t="str">
+      <x:c r="B1" s="35" t="str">
         <x:v>Authors</x:v>
       </x:c>
-      <x:c r="C1" s="18" t="str">
+      <x:c r="C1" s="35" t="str">
         <x:v>Venue</x:v>
       </x:c>
-      <x:c r="D1" s="18" t="str">
+      <x:c r="D1" s="35" t="str">
         <x:v>Venue Acronym</x:v>
       </x:c>
-      <x:c r="E1" s="18" t="str">
+      <x:c r="E1" s="35" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="18" t="str">
+      <x:c r="F1" s="35" t="str">
         <x:v>Year</x:v>
       </x:c>
-      <x:c r="G1" s="18" t="str">
+      <x:c r="G1" s="35" t="str">
         <x:v>Link</x:v>
       </x:c>
-      <x:c r="H1" s="18" t="str">
+      <x:c r="H1" s="35" t="str">
         <x:v>Bibtex</x:v>
       </x:c>
-      <x:c r="I1" s="18" t="str">
+      <x:c r="I1" s="35" t="str">
         <x:v>Abstract</x:v>
       </x:c>
-      <x:c r="J1" s="18" t="str">
+      <x:c r="J1" s="35" t="str">
         <x:v>Research Topic</x:v>
       </x:c>
-      <x:c r="K1" s="18" t="str">
+      <x:c r="K1" s="35" t="str">
         <x:v>Topic Key</x:v>
       </x:c>
     </x:row>
@@ -1281,9 +1296,9 @@
       <x:c r="F22" s="28" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G22" s="28" t="str"/>
-      <x:c r="H22" s="28" t="str"/>
-      <x:c r="I22" s="28" t="str"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="28"/>
       <x:c r="J22" s="29" t="str">
         <x:v>Adaptive, Efficient and Edge AI</x:v>
       </x:c>
@@ -1335,27 +1350,71 @@
     </x:row>
     <x:row r="24" ht="15" customHeight="1">
       <x:c r="A24" s="28" t="str">
+        <x:v>When a model is not Enough: A Complementary AI Pipeline for Ultra-Safe PCBA Defect Detection</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="str">
+        <x:v>Alberto Faro, Francesco Cancelliere, Robin Faro, Raffaele Mineo</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="str">
+        <x:v>The Autonomous Edge - Intelligence Embedded in Industrial Applications</x:v>
+      </x:c>
+      <x:c r="D24" s="28" t="str">
+        <x:v>EEAI 2025</x:v>
+      </x:c>
+      <x:c r="E24" s="28" t="str">
+        <x:v>Book Chapter</x:v>
+      </x:c>
+      <x:c r="F24" s="28" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G24" s="28" t="str">
+        <x:v>https://www.riverpublishers.com/research_details.php?book_id=1549</x:v>
+      </x:c>
+      <x:c r="H24" s="28" t="str">
+        <x:v>@incollection{faro2026when,
+  title={When a model is not Enough: A Complementary AI Pipeline for Ultra-Safe PCBA Defect Detection},
+  author={Faro, Alberto and Cancelliere, Francesco and Faro, Robin and Mineo, Raffaele},
+  booktitle={The Autonomous Edge - Intelligence Embedded in Industrial Applications},
+  editor={Vermesan, Ovidiu and Pijlman, Fetze},
+  pages={129--149},
+  year={2026},
+  publisher={River Publishers},
+  isbn={9788743815266}
+}</x:v>
+      </x:c>
+      <x:c r="I24" s="28" t="str">
+        <x:v>A multi-stage automated optical inspection pipeline for safety-critical PCBA defect detection. The approach combines a transformer optimized for high recall with specialized autoencoders that reduce false positives and residual false negatives, targeting fewer than 10 false negatives per million inspected units under a high-confidence reliability requirement. The work originates from EEAI 2025 and was published as Chapter 8 of the 2026 River Publishers volume.</x:v>
+      </x:c>
+      <x:c r="J24" s="29" t="str">
+        <x:v>Scientific and Industrial Intelligent Systems</x:v>
+      </x:c>
+      <x:c r="K24" s="29" t="str">
+        <x:v>scientific</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" customHeight="1">
+      <x:c r="A25" s="28" t="str">
         <x:v>PCB-SAID: A Low-Cost Camera-Based Dataset for Few-Shot SMD Assembly Inspection</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="str">
+      <x:c r="B25" s="28" t="str">
         <x:v>Raffaele Mineo, Amelia Sorrenti, Robin Faro, Gabriele Mineo, Francesco Cancelliere, Alberto Faro</x:v>
       </x:c>
-      <x:c r="C24" s="28" t="str">
+      <x:c r="C25" s="28" t="str">
         <x:v>Proceedings of the IEEE/CVF International Conference on Computer Vision</x:v>
       </x:c>
-      <x:c r="D24" s="28" t="str">
+      <x:c r="D25" s="28" t="str">
         <x:v>ICCV</x:v>
       </x:c>
-      <x:c r="E24" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F24" s="28" t="n">
+      <x:c r="E25" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F25" s="28" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G24" s="28" t="str">
+      <x:c r="G25" s="28" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025W/VISION%2725/html/Mineo_PCB-SAID_A_Low-Cost_Camera-Based_Dataset_for_Few-Shot_SMD_Assembly_Inspection_ICCVW_2025_paper.html</x:v>
       </x:c>
-      <x:c r="H24" s="28" t="str">
+      <x:c r="H25" s="28" t="str">
         <x:v>@inproceedings{mineo2025pcb,
   title={PCB-SAID: A Low-Cost Camera-Based Dataset for Few-Shot SMD Assembly Inspection},
   author={Mineo, Raffaele and Sorrenti, Amelia and Faro, Robin and Mineo, Gabriele and Cancelliere, Francesco and Faro, Alberto},
@@ -1364,39 +1423,39 @@
   year={2025}
 }</x:v>
       </x:c>
-      <x:c r="I24" s="28" t="str">
+      <x:c r="I25" s="28" t="str">
         <x:v>Automated Optical Inspection (AOI) of surface-mounted device (SMD) assemblies is critical for ensuring quality and yield in electronics manufacturing, yet current systems rely on expensive hardware and handcrafted algorithms that struggle with novel layouts and rare defect modes. We present PCB-SAID (Printed Circuit Board – SMD Assembly Inspection Dataset), the first open, few-shot SMD inspection dataset comprising 175 RGB images annotated with 66 fine-grained classes, spanning well-soldered, mis-soldered (misaligned, lifted, rotated), missing, and short-circuit conditions, using a rigorous two-stage expert pipeline (bounding-box localization followed by polygonal mask refinement). We evaluate five state-of-the-art architectures (Fast R-CNN, DETR, YOLOv11, YOLOv12, SAM) under both full-data and few-shot (1, 5 shots) regimes, reporting mAP@[.50:.95], mAP@.50, precision, and recall. Our results reveal optimal performance gaps on rare and subtle anomalies, underscoring challenges in class imbalance and domain shift. The dataset will be made publicly available upon request to support further research in this area.</x:v>
       </x:c>
-      <x:c r="J24" s="29" t="str">
+      <x:c r="J25" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K24" s="29" t="str">
+      <x:c r="K25" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15" customHeight="1">
-      <x:c r="A25" s="28" t="str">
+    <x:row r="26" ht="15" customHeight="1">
+      <x:c r="A26" s="28" t="str">
         <x:v>BioTrak: A Blockchain-based Platform for Food Chain Logistics Traceability</x:v>
       </x:c>
-      <x:c r="B25" s="28" t="str">
+      <x:c r="B26" s="28" t="str">
         <x:v>Alessia Spitalleri, Isaak Kavasidis, Vincenzo Cartelli, Raffaele Mineo, Francesco Rundo, Simone Palazzo, Concetto Spampinato, Daniela Giordano</x:v>
       </x:c>
-      <x:c r="C25" s="28" t="str">
+      <x:c r="C26" s="28" t="str">
         <x:v>2023 International Conference on Intelligent Computing, Communication, Networking and Services (ICCNS)</x:v>
       </x:c>
-      <x:c r="D25" s="28" t="str">
+      <x:c r="D26" s="28" t="str">
         <x:v>ICCNS</x:v>
       </x:c>
-      <x:c r="E25" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F25" s="28" t="n">
+      <x:c r="E26" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F26" s="28" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G25" s="28" t="str">
+      <x:c r="G26" s="28" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10193341</x:v>
       </x:c>
-      <x:c r="H25" s="28" t="str">
+      <x:c r="H26" s="28" t="str">
         <x:v>@inproceedings{spitalleri2023biotrak,
   title={BioTrak: A blockchain-based platform for food chain logistics traceability},
   author={Spitalleri, Alessia and Kavasidis, Isaak and Cartelli, Vincenzo and Mineo, Raffaele and Rundo, Francesco and Palazzo, Simone and Spampinato, Concetto and Giordano, Daniela},
@@ -1406,39 +1465,39 @@
   organization={IEEE}
 }</x:v>
       </x:c>
-      <x:c r="I25" s="28" t="str">
+      <x:c r="I26" s="28" t="str">
         <x:v>The food supply chain, following its globalization, has become very complex. Such complexities, introduce factors that influence adversely the quality of intermediate and final products. Strict constraints regarding parameters such as maintenance temperatures and transportation times must be respected in order to ensure top quality and reduce to a minimum the detrimental effects to public health. This is a multi-factorial endeavor and all of the involved stakeholders must accept and manage the logistics burden to achieve the best possible results.However, such burden comes together with additional complexities and costs regarding data storage, business process management and company specific standard operating procedures and as such, automated methods must be devised to reduce the impact of such intrusive operations.For the above reasons, in this paper we present BioTrak: a platform capable of registering and visualizing the whole chain of transformation and transportation processes including the monitoring of cold chain logistics of food ingredients starting from the raw material producers until the final product arrives to the end-consumer.The platform includes Business Process Modelling methods to aid food supply chain stakeholders to optimize their processes and also integrates a blockchain for guaranteeing the integrity, transparency and accountability of the data.</x:v>
       </x:c>
-      <x:c r="J25" s="29" t="str">
+      <x:c r="J26" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K25" s="29" t="str">
+      <x:c r="K26" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15" customHeight="1">
-      <x:c r="A26" s="28" t="str">
+    <x:row r="27" ht="15" customHeight="1">
+      <x:c r="A27" s="28" t="str">
         <x:v>EUROVOLC - Deliverable Report - D9.3 Machine learning tool kit and database</x:v>
       </x:c>
-      <x:c r="B26" s="28" t="str">
+      <x:c r="B27" s="28" t="str">
         <x:v>S. Palazzo, R. Mineo, C. Spampinato, F. Cannavò, A. Cannata, C. Montagna, J. M. Saurel, O. Geber, A. Lemarchand</x:v>
       </x:c>
-      <x:c r="C26" s="28" t="str">
+      <x:c r="C27" s="28" t="str">
         <x:v>HORIZON 2020 EUROVOLC Project</x:v>
       </x:c>
-      <x:c r="D26" s="28" t="str">
+      <x:c r="D27" s="28" t="str">
         <x:v>EUROVOLC</x:v>
       </x:c>
-      <x:c r="E26" s="28" t="str">
+      <x:c r="E27" s="28" t="str">
         <x:v>Project</x:v>
       </x:c>
-      <x:c r="F26" s="28" t="n">
+      <x:c r="F27" s="28" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G26" s="28" t="str">
+      <x:c r="G27" s="28" t="str">
         <x:v>https://eurovolc.eu/wp-content/uploads/2021/08/D9.3.pdf</x:v>
       </x:c>
-      <x:c r="H26" s="28" t="str">
+      <x:c r="H27" s="28" t="str">
         <x:v>@techreport{palazzo2021eurovolc_d93,
   title={Machine learning tool kit and database},
   author={Palazzo, Simone and Mineo, Raffaele and Spampinato, Concetto and Cannav{\`o}, Flavio and Cannata, Andrea and Montagna, Chiara and Saurel, Jean-Marie and Geber, O. and Lemarchand, Arnaud},
@@ -1448,39 +1507,39 @@
   note={Horizon 2020 {EUROVOLC}, Grant Agreement No. 731070}
 }</x:v>
       </x:c>
-      <x:c r="I26" s="28" t="str">
+      <x:c r="I27" s="28" t="str">
         <x:v>The recent success of deep learning techniques has stimulated the application of such approaches for the automatic identification of models related to volcanic phenomena. In this study, a tool was developed for anomaly detection in historical volcanic data in an unsupervised manner. The results on data from Etna and Stromboli are promising, highlighting the ability to anticipate significant anomalies with respect to volcanic events.</x:v>
       </x:c>
-      <x:c r="J26" s="29" t="str">
+      <x:c r="J27" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K26" s="29" t="str">
+      <x:c r="K27" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15" customHeight="1">
-      <x:c r="A27" s="28" t="str">
+    <x:row r="28" ht="15" customHeight="1">
+      <x:c r="A28" s="28" t="str">
         <x:v>VOLcano UNrest Detection (VolUnD) Toolkit</x:v>
       </x:c>
-      <x:c r="B27" s="28" t="str">
+      <x:c r="B28" s="28" t="str">
         <x:v>R. Mineo, P. Spadaro, F. Cannavò, S. Palazzo, A. Cannata, C. Spampinato</x:v>
       </x:c>
-      <x:c r="C27" s="28" t="str">
+      <x:c r="C28" s="28" t="str">
         <x:v>Zenodo</x:v>
       </x:c>
-      <x:c r="D27" s="28" t="str">
+      <x:c r="D28" s="28" t="str">
         <x:v>Zenodo</x:v>
       </x:c>
-      <x:c r="E27" s="28" t="str">
+      <x:c r="E28" s="28" t="str">
         <x:v>Software</x:v>
       </x:c>
-      <x:c r="F27" s="28" t="n">
+      <x:c r="F28" s="28" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G27" s="28" t="str">
+      <x:c r="G28" s="30" t="str">
         <x:v>https://zenodo.org/records/5541125</x:v>
       </x:c>
-      <x:c r="H27" s="28" t="str">
+      <x:c r="H28" s="30" t="str">
         <x:v>@misc{raffaele_mineo_2021_5541125,
   title={EUROVOLC-ML/VolUnD-Toolkit: VolUnD v1.0},
   author={Mineo, Raffaele and Spadaro, Paolo and Cannav{\`o}, Flavio and Palazzo, Simone and Cannata, Andrea and Spampinato, Concetto},
@@ -1489,39 +1548,39 @@
   doi={10.5281/zenodo.5541125}
 }</x:v>
       </x:c>
-      <x:c r="I27" s="28" t="str">
+      <x:c r="I28" s="28" t="str">
         <x:v>VolUnD is a VOLcano UNrest Detection toolkit written in (PyTorch) Python. Performs anomaly detection of historical volcanic data in an unsupervised manner, leveraging the hypothesis that normal activity dominates the distribution of events and can therefore be treated as the main source of information for training a model capable of identifying deviations as anomalies. These anomalies could be attributed to changes in the state of the volcano.</x:v>
       </x:c>
-      <x:c r="J27" s="29" t="str">
+      <x:c r="J28" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K27" s="29" t="str">
+      <x:c r="K28" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" customHeight="1">
-      <x:c r="A28" s="28" t="str">
+    <x:row r="29" ht="15" customHeight="1">
+      <x:c r="A29" s="28" t="str">
         <x:v>Advancing Healthcare with Multimodal AI: Enhanced Diagnosis, Cognitive Monitoring, and Inclusive Medical Communication</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="str">
+      <x:c r="B29" s="28" t="str">
         <x:v>Raffaele Mineo</x:v>
       </x:c>
-      <x:c r="C28" s="28" t="str">
+      <x:c r="C29" s="28" t="str">
         <x:v>International Conference on Medical Image Computing and Computer-Assisted Intervention</x:v>
       </x:c>
-      <x:c r="D28" s="28" t="str">
+      <x:c r="D29" s="28" t="str">
         <x:v>MICCAI</x:v>
       </x:c>
-      <x:c r="E28" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F28" s="28" t="n">
+      <x:c r="E29" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F29" s="28" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="G28" s="30" t="str">
+      <x:c r="G29" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="H28" s="30" t="str">
+      <x:c r="H29" s="28" t="str">
         <x:v>@inproceedings{mineo2025advancing,
   title={Advancing Healthcare with Multimodal AI: Enhanced Diagnosis, Cognitive Monitoring, and Inclusive Medical Communication},
   author={Mineo, Raffaele},
@@ -1530,39 +1589,39 @@
   organization={Springer}
 }</x:v>
       </x:c>
-      <x:c r="I28" s="28" t="str">
+      <x:c r="I29" s="28" t="str">
         <x:v>This doctoral research explores multimodal deep learning to enhance diagnosis, cognitive monitoring, and communication accessibility in healthcare. Across three clinical domains - cardiovascular diagnostics, neurocognitive assessment, and sign language recognition - we develop transformer-based pipelines tailored for real-time applicability, interpretability, and privacy compliance. In the cardiovascular setting, we propose spatio-temporal models for non-invasive estimation of FFR and iFR from single-view coronary angiography, integrating convolutional and transformer encoders with multi-task supervision. These innovations culminate in the STARFLOW system, a deployable platform achieving high accuracy in multicenter studies, and protected by national and EU patents. For cognitive screening, we introduce pipelines that analyze facial micro-movements and eye-gaze trajectories using phase-based motion magnification, attention-based encoders, and a novel Time-Aware Positional Embedding (TAPE) module. These systems enable automated scoring of MMSE and MoCA using commodity tablets, facilitating contactless and scalable cognitive health tools. To promote inclusivity, we release MultiMedaLIS, the first multimodal dataset of Italian medical sign language, and develop a GDPR-compliant radar-based recognition pipeline using Range-Doppler Maps and temporal transformers. This system ensures robust gesture classification under privacy and environmental constraints. Collectively, this work contributes a unified framework for interpretable and adaptive AI in healthcare, advancing real-world integration through methodological innovation, validated deployment, and alignment with clinical needs.</x:v>
       </x:c>
-      <x:c r="J28" s="29" t="str">
+      <x:c r="J29" s="29" t="str">
         <x:v>Research Synthesis and Scholarly Outputs</x:v>
       </x:c>
-      <x:c r="K28" s="29" t="str">
+      <x:c r="K29" s="29" t="str">
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="15" customHeight="1">
-      <x:c r="A29" s="28" t="str">
+    <x:row r="30">
+      <x:c r="A30" s="29" t="str">
         <x:v>Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25)</x:v>
       </x:c>
-      <x:c r="B29" s="28" t="str">
+      <x:c r="B30" s="29" t="str">
         <x:v>Simone Palazzo, Giovanni Bellitto, Raffaele Mineo, Amelia Sorrenti, Camila Gonzalez, Angelo Porrello, Lorenzo Bonicelli</x:v>
       </x:c>
-      <x:c r="C29" s="28" t="str">
+      <x:c r="C30" s="29" t="str">
         <x:v>ACM Multimedia 2025</x:v>
       </x:c>
-      <x:c r="D29" s="28" t="str">
+      <x:c r="D30" s="29" t="str">
         <x:v>ACM MM</x:v>
       </x:c>
-      <x:c r="E29" s="28" t="str">
+      <x:c r="E30" s="29" t="str">
         <x:v>Edited Proceedings</x:v>
       </x:c>
-      <x:c r="F29" s="28" t="n">
+      <x:c r="F30" s="29" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G29" s="28" t="str">
+      <x:c r="G30" s="29" t="str">
         <x:v>https://dl.acm.org/doi/pdf/10.1145/3746259</x:v>
       </x:c>
-      <x:c r="H29" s="28" t="str">
+      <x:c r="H30" s="29" t="str">
         <x:v>@proceedings{pilm2025,
   title={Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25), co-located with ACM Multimedia 2025},
   editor={Palazzo, Simone and Bellitto, Giovanni and Mineo, Raffaele and Sorrenti, Amelia and Gonzalez, Camila and Porrello, Angelo and Bonicelli, Lorenzo},
@@ -1571,20 +1630,20 @@
   doi={10.1145/3746259}
 }</x:v>
       </x:c>
-      <x:c r="I29" s="28" t="str">
+      <x:c r="I30" s="29" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="J29" s="29" t="str">
+      <x:c r="J30" s="29" t="str">
         <x:v>Research Synthesis and Scholarly Outputs</x:v>
       </x:c>
-      <x:c r="K29" s="29" t="str">
+      <x:c r="K30" s="29" t="str">
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff2b2d6788ce4bb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4c8eb9bea614051"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Preserve publication metadata row styling
</commit_message>
<xml_diff>
--- a/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
+++ b/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="Rb48d95a0360b4a68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="R0019d453500c4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R5bd02afd9028415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="Rfb6e92ca843a47dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,7 +32,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -49,6 +49,11 @@
         <x:fgColor rgb="FF0B1F33"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB4E6A2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -57,7 +62,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -151,12 +156,21 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normale" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="11">
+  <x:dxfs count="13">
     <x:dxf/>
     <x:dxf/>
     <x:dxf/>
@@ -168,6 +182,20 @@
     <x:dxf/>
     <x:dxf/>
     <x:dxf/>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFB4E6A2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9F2D0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -1599,29 +1627,29 @@
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="29" t="str">
+    <x:row r="30" ht="15" customHeight="1">
+      <x:c r="A30" s="37" t="str">
         <x:v>Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25)</x:v>
       </x:c>
-      <x:c r="B30" s="29" t="str">
+      <x:c r="B30" s="37" t="str">
         <x:v>Simone Palazzo, Giovanni Bellitto, Raffaele Mineo, Amelia Sorrenti, Camila Gonzalez, Angelo Porrello, Lorenzo Bonicelli</x:v>
       </x:c>
-      <x:c r="C30" s="29" t="str">
+      <x:c r="C30" s="37" t="str">
         <x:v>ACM Multimedia 2025</x:v>
       </x:c>
-      <x:c r="D30" s="29" t="str">
+      <x:c r="D30" s="37" t="str">
         <x:v>ACM MM</x:v>
       </x:c>
-      <x:c r="E30" s="29" t="str">
+      <x:c r="E30" s="37" t="str">
         <x:v>Edited Proceedings</x:v>
       </x:c>
-      <x:c r="F30" s="29" t="n">
+      <x:c r="F30" s="37" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G30" s="29" t="str">
+      <x:c r="G30" s="37" t="str">
         <x:v>https://dl.acm.org/doi/pdf/10.1145/3746259</x:v>
       </x:c>
-      <x:c r="H30" s="29" t="str">
+      <x:c r="H30" s="37" t="str">
         <x:v>@proceedings{pilm2025,
   title={Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25), co-located with ACM Multimedia 2025},
   editor={Palazzo, Simone and Bellitto, Giovanni and Mineo, Raffaele and Sorrenti, Amelia and Gonzalez, Camila and Porrello, Angelo and Bonicelli, Lorenzo},
@@ -1630,20 +1658,498 @@
   doi={10.1145/3746259}
 }</x:v>
       </x:c>
-      <x:c r="I30" s="29" t="str">
+      <x:c r="I30" s="37" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="J30" s="29" t="str">
+      <x:c r="J30" s="38" t="str">
         <x:v>Research Synthesis and Scholarly Outputs</x:v>
       </x:c>
-      <x:c r="K30" s="29" t="str">
+      <x:c r="K30" s="38" t="str">
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="15" customHeight="1"/>
+    <x:row r="32" ht="15" customHeight="1"/>
+    <x:row r="33" ht="15" customHeight="1"/>
+    <x:row r="34" ht="15" customHeight="1"/>
+    <x:row r="35" ht="15" customHeight="1"/>
+    <x:row r="36" ht="15" customHeight="1"/>
+    <x:row r="37" ht="15" customHeight="1"/>
+    <x:row r="38" ht="15" customHeight="1"/>
+    <x:row r="39" ht="15" customHeight="1"/>
+    <x:row r="40" ht="15" customHeight="1"/>
+    <x:row r="41" ht="15" customHeight="1"/>
+    <x:row r="42" ht="15" customHeight="1"/>
+    <x:row r="43" ht="15" customHeight="1"/>
+    <x:row r="44" ht="15" customHeight="1"/>
+    <x:row r="45" ht="15" customHeight="1"/>
+    <x:row r="46" ht="15" customHeight="1"/>
+    <x:row r="47" ht="15" customHeight="1"/>
+    <x:row r="48" ht="15" customHeight="1"/>
+    <x:row r="49" ht="15" customHeight="1"/>
+    <x:row r="50" ht="15" customHeight="1"/>
+    <x:row r="51" ht="15" customHeight="1"/>
+    <x:row r="52" ht="15" customHeight="1"/>
+    <x:row r="53" ht="15" customHeight="1"/>
+    <x:row r="54" ht="15" customHeight="1"/>
+    <x:row r="55" ht="15" customHeight="1"/>
+    <x:row r="56" ht="15" customHeight="1"/>
+    <x:row r="57" ht="15" customHeight="1"/>
+    <x:row r="58" ht="15" customHeight="1"/>
+    <x:row r="59" ht="15" customHeight="1"/>
+    <x:row r="60" ht="15" customHeight="1"/>
+    <x:row r="61" ht="15" customHeight="1"/>
+    <x:row r="62" ht="15" customHeight="1"/>
+    <x:row r="63" ht="15" customHeight="1"/>
+    <x:row r="64" ht="15" customHeight="1"/>
+    <x:row r="65" ht="15" customHeight="1"/>
+    <x:row r="66" ht="15" customHeight="1"/>
+    <x:row r="67" ht="15" customHeight="1"/>
+    <x:row r="68" ht="15" customHeight="1"/>
+    <x:row r="69" ht="15" customHeight="1"/>
+    <x:row r="70" ht="15" customHeight="1"/>
+    <x:row r="71" ht="15" customHeight="1"/>
+    <x:row r="72" ht="15" customHeight="1"/>
+    <x:row r="73" ht="15" customHeight="1"/>
+    <x:row r="74" ht="15" customHeight="1"/>
+    <x:row r="75" ht="15" customHeight="1"/>
+    <x:row r="76" ht="15" customHeight="1"/>
+    <x:row r="77" ht="15" customHeight="1"/>
+    <x:row r="78" ht="15" customHeight="1"/>
+    <x:row r="79" ht="15" customHeight="1"/>
+    <x:row r="80" ht="15" customHeight="1"/>
+    <x:row r="81" ht="15" customHeight="1"/>
+    <x:row r="82" ht="15" customHeight="1"/>
+    <x:row r="83" ht="15" customHeight="1"/>
+    <x:row r="84" ht="15" customHeight="1"/>
+    <x:row r="85" ht="15" customHeight="1"/>
+    <x:row r="86" ht="15" customHeight="1"/>
+    <x:row r="87" ht="15" customHeight="1"/>
+    <x:row r="88" ht="15" customHeight="1"/>
+    <x:row r="89" ht="15" customHeight="1"/>
+    <x:row r="90" ht="15" customHeight="1"/>
+    <x:row r="91" ht="15" customHeight="1"/>
+    <x:row r="92" ht="15" customHeight="1"/>
+    <x:row r="93" ht="15" customHeight="1"/>
+    <x:row r="94" ht="15" customHeight="1"/>
+    <x:row r="95" ht="15" customHeight="1"/>
+    <x:row r="96" ht="15" customHeight="1"/>
+    <x:row r="97" ht="15" customHeight="1"/>
+    <x:row r="98" ht="15" customHeight="1"/>
+    <x:row r="99" ht="15" customHeight="1"/>
+    <x:row r="100" ht="15" customHeight="1"/>
+    <x:row r="101" ht="15" customHeight="1"/>
+    <x:row r="102" ht="15" customHeight="1"/>
+    <x:row r="103" ht="15" customHeight="1"/>
+    <x:row r="104" ht="15" customHeight="1"/>
+    <x:row r="105" ht="15" customHeight="1"/>
+    <x:row r="106" ht="15" customHeight="1"/>
+    <x:row r="107" ht="15" customHeight="1"/>
+    <x:row r="108" ht="15" customHeight="1"/>
+    <x:row r="109" ht="15" customHeight="1"/>
+    <x:row r="110" ht="15" customHeight="1"/>
+    <x:row r="111" ht="15" customHeight="1"/>
+    <x:row r="112" ht="15" customHeight="1"/>
+    <x:row r="113" ht="15" customHeight="1"/>
+    <x:row r="114" ht="15" customHeight="1"/>
+    <x:row r="115" ht="15" customHeight="1"/>
+    <x:row r="116" ht="15" customHeight="1"/>
+    <x:row r="117" ht="15" customHeight="1"/>
+    <x:row r="118" ht="15" customHeight="1"/>
+    <x:row r="119" ht="15" customHeight="1"/>
+    <x:row r="120" ht="15" customHeight="1"/>
+    <x:row r="121" ht="15" customHeight="1"/>
+    <x:row r="122" ht="15" customHeight="1"/>
+    <x:row r="123" ht="15" customHeight="1"/>
+    <x:row r="124" ht="15" customHeight="1"/>
+    <x:row r="125" ht="15" customHeight="1"/>
+    <x:row r="126" ht="15" customHeight="1"/>
+    <x:row r="127" ht="15" customHeight="1"/>
+    <x:row r="128" ht="15" customHeight="1"/>
+    <x:row r="129" ht="15" customHeight="1"/>
+    <x:row r="130" ht="15" customHeight="1"/>
+    <x:row r="131" ht="15" customHeight="1"/>
+    <x:row r="132" ht="15" customHeight="1"/>
+    <x:row r="133" ht="15" customHeight="1"/>
+    <x:row r="134" ht="15" customHeight="1"/>
+    <x:row r="135" ht="15" customHeight="1"/>
+    <x:row r="136" ht="15" customHeight="1"/>
+    <x:row r="137" ht="15" customHeight="1"/>
+    <x:row r="138" ht="15" customHeight="1"/>
+    <x:row r="139" ht="15" customHeight="1"/>
+    <x:row r="140" ht="15" customHeight="1"/>
+    <x:row r="141" ht="15" customHeight="1"/>
+    <x:row r="142" ht="15" customHeight="1"/>
+    <x:row r="143" ht="15" customHeight="1"/>
+    <x:row r="144" ht="15" customHeight="1"/>
+    <x:row r="145" ht="15" customHeight="1"/>
+    <x:row r="146" ht="15" customHeight="1"/>
+    <x:row r="147" ht="15" customHeight="1"/>
+    <x:row r="148" ht="15" customHeight="1"/>
+    <x:row r="149" ht="15" customHeight="1"/>
+    <x:row r="150" ht="15" customHeight="1"/>
+    <x:row r="151" ht="15" customHeight="1"/>
+    <x:row r="152" ht="15" customHeight="1"/>
+    <x:row r="153" ht="15" customHeight="1"/>
+    <x:row r="154" ht="15" customHeight="1"/>
+    <x:row r="155" ht="15" customHeight="1"/>
+    <x:row r="156" ht="15" customHeight="1"/>
+    <x:row r="157" ht="15" customHeight="1"/>
+    <x:row r="158" ht="15" customHeight="1"/>
+    <x:row r="159" ht="15" customHeight="1"/>
+    <x:row r="160" ht="15" customHeight="1"/>
+    <x:row r="161" ht="15" customHeight="1"/>
+    <x:row r="162" ht="15" customHeight="1"/>
+    <x:row r="163" ht="15" customHeight="1"/>
+    <x:row r="164" ht="15" customHeight="1"/>
+    <x:row r="165" ht="15" customHeight="1"/>
+    <x:row r="166" ht="15" customHeight="1"/>
+    <x:row r="167" ht="15" customHeight="1"/>
+    <x:row r="168" ht="15" customHeight="1"/>
+    <x:row r="169" ht="15" customHeight="1"/>
+    <x:row r="170" ht="15" customHeight="1"/>
+    <x:row r="171" ht="15" customHeight="1"/>
+    <x:row r="172" ht="15" customHeight="1"/>
+    <x:row r="173" ht="15" customHeight="1"/>
+    <x:row r="174" ht="15" customHeight="1"/>
+    <x:row r="175" ht="15" customHeight="1"/>
+    <x:row r="176" ht="15" customHeight="1"/>
+    <x:row r="177" ht="15" customHeight="1"/>
+    <x:row r="178" ht="15" customHeight="1"/>
+    <x:row r="179" ht="15" customHeight="1"/>
+    <x:row r="180" ht="15" customHeight="1"/>
+    <x:row r="181" ht="15" customHeight="1"/>
+    <x:row r="182" ht="15" customHeight="1"/>
+    <x:row r="183" ht="15" customHeight="1"/>
+    <x:row r="184" ht="15" customHeight="1"/>
+    <x:row r="185" ht="15" customHeight="1"/>
+    <x:row r="186" ht="15" customHeight="1"/>
+    <x:row r="187" ht="15" customHeight="1"/>
+    <x:row r="188" ht="15" customHeight="1"/>
+    <x:row r="189" ht="15" customHeight="1"/>
+    <x:row r="190" ht="15" customHeight="1"/>
+    <x:row r="191" ht="15" customHeight="1"/>
+    <x:row r="192" ht="15" customHeight="1"/>
+    <x:row r="193" ht="15" customHeight="1"/>
+    <x:row r="194" ht="15" customHeight="1"/>
+    <x:row r="195" ht="15" customHeight="1"/>
+    <x:row r="196" ht="15" customHeight="1"/>
+    <x:row r="197" ht="15" customHeight="1"/>
+    <x:row r="198" ht="15" customHeight="1"/>
+    <x:row r="199" ht="15" customHeight="1"/>
+    <x:row r="200" ht="15" customHeight="1"/>
+    <x:row r="201" ht="15" customHeight="1"/>
+    <x:row r="202" ht="15" customHeight="1"/>
+    <x:row r="203" ht="15" customHeight="1"/>
+    <x:row r="204" ht="15" customHeight="1"/>
+    <x:row r="205" ht="15" customHeight="1"/>
+    <x:row r="206" ht="15" customHeight="1"/>
+    <x:row r="207" ht="15" customHeight="1"/>
+    <x:row r="208" ht="15" customHeight="1"/>
+    <x:row r="209" ht="15" customHeight="1"/>
+    <x:row r="210" ht="15" customHeight="1"/>
+    <x:row r="211" ht="15" customHeight="1"/>
+    <x:row r="212" ht="15" customHeight="1"/>
+    <x:row r="213" ht="15" customHeight="1"/>
+    <x:row r="214" ht="15" customHeight="1"/>
+    <x:row r="215" ht="15" customHeight="1"/>
+    <x:row r="216" ht="15" customHeight="1"/>
+    <x:row r="217" ht="15" customHeight="1"/>
+    <x:row r="218" ht="15" customHeight="1"/>
+    <x:row r="219" ht="15" customHeight="1"/>
+    <x:row r="220" ht="15" customHeight="1"/>
+    <x:row r="221" ht="15" customHeight="1"/>
+    <x:row r="222" ht="15" customHeight="1"/>
+    <x:row r="223" ht="15" customHeight="1"/>
+    <x:row r="224" ht="15" customHeight="1"/>
+    <x:row r="225" ht="15" customHeight="1"/>
+    <x:row r="226" ht="15" customHeight="1"/>
+    <x:row r="227" ht="15" customHeight="1"/>
+    <x:row r="228" ht="15" customHeight="1"/>
+    <x:row r="229" ht="15" customHeight="1"/>
+    <x:row r="230" ht="15" customHeight="1"/>
+    <x:row r="231" ht="15" customHeight="1"/>
+    <x:row r="232" ht="15" customHeight="1"/>
+    <x:row r="233" ht="15" customHeight="1"/>
+    <x:row r="234" ht="15" customHeight="1"/>
+    <x:row r="235" ht="15" customHeight="1"/>
+    <x:row r="236" ht="15" customHeight="1"/>
+    <x:row r="237" ht="15" customHeight="1"/>
+    <x:row r="238" ht="15" customHeight="1"/>
+    <x:row r="239" ht="15" customHeight="1"/>
+    <x:row r="240" ht="15" customHeight="1"/>
+    <x:row r="241" ht="15" customHeight="1"/>
+    <x:row r="242" ht="15" customHeight="1"/>
+    <x:row r="243" ht="15" customHeight="1"/>
+    <x:row r="244" ht="15" customHeight="1"/>
+    <x:row r="245" ht="15" customHeight="1"/>
+    <x:row r="246" ht="15" customHeight="1"/>
+    <x:row r="247" ht="15" customHeight="1"/>
+    <x:row r="248" ht="15" customHeight="1"/>
+    <x:row r="249" ht="15" customHeight="1"/>
+    <x:row r="250" ht="15" customHeight="1"/>
+    <x:row r="251" ht="15" customHeight="1"/>
+    <x:row r="252" ht="15" customHeight="1"/>
+    <x:row r="253" ht="15" customHeight="1"/>
+    <x:row r="254" ht="15" customHeight="1"/>
+    <x:row r="255" ht="15" customHeight="1"/>
+    <x:row r="256" ht="15" customHeight="1"/>
+    <x:row r="257" ht="15" customHeight="1"/>
+    <x:row r="258" ht="15" customHeight="1"/>
+    <x:row r="259" ht="15" customHeight="1"/>
+    <x:row r="260" ht="15" customHeight="1"/>
+    <x:row r="261" ht="15" customHeight="1"/>
+    <x:row r="262" ht="15" customHeight="1"/>
+    <x:row r="263" ht="15" customHeight="1"/>
+    <x:row r="264" ht="15" customHeight="1"/>
+    <x:row r="265" ht="15" customHeight="1"/>
+    <x:row r="266" ht="15" customHeight="1"/>
+    <x:row r="267" ht="15" customHeight="1"/>
+    <x:row r="268" ht="15" customHeight="1"/>
+    <x:row r="269" ht="15" customHeight="1"/>
+    <x:row r="270" ht="15" customHeight="1"/>
+    <x:row r="271" ht="15" customHeight="1"/>
+    <x:row r="272" ht="15" customHeight="1"/>
+    <x:row r="273" ht="15" customHeight="1"/>
+    <x:row r="274" ht="15" customHeight="1"/>
+    <x:row r="275" ht="15" customHeight="1"/>
+    <x:row r="276" ht="15" customHeight="1"/>
+    <x:row r="277" ht="15" customHeight="1"/>
+    <x:row r="278" ht="15" customHeight="1"/>
+    <x:row r="279" ht="15" customHeight="1"/>
+    <x:row r="280" ht="15" customHeight="1"/>
+    <x:row r="281" ht="15" customHeight="1"/>
+    <x:row r="282" ht="15" customHeight="1"/>
+    <x:row r="283" ht="15" customHeight="1"/>
+    <x:row r="284" ht="15" customHeight="1"/>
+    <x:row r="285" ht="15" customHeight="1"/>
+    <x:row r="286" ht="15" customHeight="1"/>
+    <x:row r="287" ht="15" customHeight="1"/>
+    <x:row r="288" ht="15" customHeight="1"/>
+    <x:row r="289" ht="15" customHeight="1"/>
+    <x:row r="290" ht="15" customHeight="1"/>
+    <x:row r="291" ht="15" customHeight="1"/>
+    <x:row r="292" ht="15" customHeight="1"/>
+    <x:row r="293" ht="15" customHeight="1"/>
+    <x:row r="294" ht="15" customHeight="1"/>
+    <x:row r="295" ht="15" customHeight="1"/>
+    <x:row r="296" ht="15" customHeight="1"/>
+    <x:row r="297" ht="15" customHeight="1"/>
+    <x:row r="298" ht="15" customHeight="1"/>
+    <x:row r="299" ht="15" customHeight="1"/>
+    <x:row r="300" ht="15" customHeight="1"/>
+    <x:row r="301" ht="15" customHeight="1"/>
+    <x:row r="302" ht="15" customHeight="1"/>
+    <x:row r="303" ht="15" customHeight="1"/>
+    <x:row r="304" ht="15" customHeight="1"/>
+    <x:row r="305" ht="15" customHeight="1"/>
+    <x:row r="306" ht="15" customHeight="1"/>
+    <x:row r="307" ht="15" customHeight="1"/>
+    <x:row r="308" ht="15" customHeight="1"/>
+    <x:row r="309" ht="15" customHeight="1"/>
+    <x:row r="310" ht="15" customHeight="1"/>
+    <x:row r="311" ht="15" customHeight="1"/>
+    <x:row r="312" ht="15" customHeight="1"/>
+    <x:row r="313" ht="15" customHeight="1"/>
+    <x:row r="314" ht="15" customHeight="1"/>
+    <x:row r="315" ht="15" customHeight="1"/>
+    <x:row r="316" ht="15" customHeight="1"/>
+    <x:row r="317" ht="15" customHeight="1"/>
+    <x:row r="318" ht="15" customHeight="1"/>
+    <x:row r="319" ht="15" customHeight="1"/>
+    <x:row r="320" ht="15" customHeight="1"/>
+    <x:row r="321" ht="15" customHeight="1"/>
+    <x:row r="322" ht="15" customHeight="1"/>
+    <x:row r="323" ht="15" customHeight="1"/>
+    <x:row r="324" ht="15" customHeight="1"/>
+    <x:row r="325" ht="15" customHeight="1"/>
+    <x:row r="326" ht="15" customHeight="1"/>
+    <x:row r="327" ht="15" customHeight="1"/>
+    <x:row r="328" ht="15" customHeight="1"/>
+    <x:row r="329" ht="15" customHeight="1"/>
+    <x:row r="330" ht="15" customHeight="1"/>
+    <x:row r="331" ht="15" customHeight="1"/>
+    <x:row r="332" ht="15" customHeight="1"/>
+    <x:row r="333" ht="15" customHeight="1"/>
+    <x:row r="334" ht="15" customHeight="1"/>
+    <x:row r="335" ht="15" customHeight="1"/>
+    <x:row r="336" ht="15" customHeight="1"/>
+    <x:row r="337" ht="15" customHeight="1"/>
+    <x:row r="338" ht="15" customHeight="1"/>
+    <x:row r="339" ht="15" customHeight="1"/>
+    <x:row r="340" ht="15" customHeight="1"/>
+    <x:row r="341" ht="15" customHeight="1"/>
+    <x:row r="342" ht="15" customHeight="1"/>
+    <x:row r="343" ht="15" customHeight="1"/>
+    <x:row r="344" ht="15" customHeight="1"/>
+    <x:row r="345" ht="15" customHeight="1"/>
+    <x:row r="346" ht="15" customHeight="1"/>
+    <x:row r="347" ht="15" customHeight="1"/>
+    <x:row r="348" ht="15" customHeight="1"/>
+    <x:row r="349" ht="15" customHeight="1"/>
+    <x:row r="350" ht="15" customHeight="1"/>
+    <x:row r="351" ht="15" customHeight="1"/>
+    <x:row r="352" ht="15" customHeight="1"/>
+    <x:row r="353" ht="15" customHeight="1"/>
+    <x:row r="354" ht="15" customHeight="1"/>
+    <x:row r="355" ht="15" customHeight="1"/>
+    <x:row r="356" ht="15" customHeight="1"/>
+    <x:row r="357" ht="15" customHeight="1"/>
+    <x:row r="358" ht="15" customHeight="1"/>
+    <x:row r="359" ht="15" customHeight="1"/>
+    <x:row r="360" ht="15" customHeight="1"/>
+    <x:row r="361" ht="15" customHeight="1"/>
+    <x:row r="362" ht="15" customHeight="1"/>
+    <x:row r="363" ht="15" customHeight="1"/>
+    <x:row r="364" ht="15" customHeight="1"/>
+    <x:row r="365" ht="15" customHeight="1"/>
+    <x:row r="366" ht="15" customHeight="1"/>
+    <x:row r="367" ht="15" customHeight="1"/>
+    <x:row r="368" ht="15" customHeight="1"/>
+    <x:row r="369" ht="15" customHeight="1"/>
+    <x:row r="370" ht="15" customHeight="1"/>
+    <x:row r="371" ht="15" customHeight="1"/>
+    <x:row r="372" ht="15" customHeight="1"/>
+    <x:row r="373" ht="15" customHeight="1"/>
+    <x:row r="374" ht="15" customHeight="1"/>
+    <x:row r="375" ht="15" customHeight="1"/>
+    <x:row r="376" ht="15" customHeight="1"/>
+    <x:row r="377" ht="15" customHeight="1"/>
+    <x:row r="378" ht="15" customHeight="1"/>
+    <x:row r="379" ht="15" customHeight="1"/>
+    <x:row r="380" ht="15" customHeight="1"/>
+    <x:row r="381" ht="15" customHeight="1"/>
+    <x:row r="382" ht="15" customHeight="1"/>
+    <x:row r="383" ht="15" customHeight="1"/>
+    <x:row r="384" ht="15" customHeight="1"/>
+    <x:row r="385" ht="15" customHeight="1"/>
+    <x:row r="386" ht="15" customHeight="1"/>
+    <x:row r="387" ht="15" customHeight="1"/>
+    <x:row r="388" ht="15" customHeight="1"/>
+    <x:row r="389" ht="15" customHeight="1"/>
+    <x:row r="390" ht="15" customHeight="1"/>
+    <x:row r="391" ht="15" customHeight="1"/>
+    <x:row r="392" ht="15" customHeight="1"/>
+    <x:row r="393" ht="15" customHeight="1"/>
+    <x:row r="394" ht="15" customHeight="1"/>
+    <x:row r="395" ht="15" customHeight="1"/>
+    <x:row r="396" ht="15" customHeight="1"/>
+    <x:row r="397" ht="15" customHeight="1"/>
+    <x:row r="398" ht="15" customHeight="1"/>
+    <x:row r="399" ht="15" customHeight="1"/>
+    <x:row r="400" ht="15" customHeight="1"/>
+    <x:row r="401" ht="15" customHeight="1"/>
+    <x:row r="402" ht="15" customHeight="1"/>
+    <x:row r="403" ht="15" customHeight="1"/>
+    <x:row r="404" ht="15" customHeight="1"/>
+    <x:row r="405" ht="15" customHeight="1"/>
+    <x:row r="406" ht="15" customHeight="1"/>
+    <x:row r="407" ht="15" customHeight="1"/>
+    <x:row r="408" ht="15" customHeight="1"/>
+    <x:row r="409" ht="15" customHeight="1"/>
+    <x:row r="410" ht="15" customHeight="1"/>
+    <x:row r="411" ht="15" customHeight="1"/>
+    <x:row r="412" ht="15" customHeight="1"/>
+    <x:row r="413" ht="15" customHeight="1"/>
+    <x:row r="414" ht="15" customHeight="1"/>
+    <x:row r="415" ht="15" customHeight="1"/>
+    <x:row r="416" ht="15" customHeight="1"/>
+    <x:row r="417" ht="15" customHeight="1"/>
+    <x:row r="418" ht="15" customHeight="1"/>
+    <x:row r="419" ht="15" customHeight="1"/>
+    <x:row r="420" ht="15" customHeight="1"/>
+    <x:row r="421" ht="15" customHeight="1"/>
+    <x:row r="422" ht="15" customHeight="1"/>
+    <x:row r="423" ht="15" customHeight="1"/>
+    <x:row r="424" ht="15" customHeight="1"/>
+    <x:row r="425" ht="15" customHeight="1"/>
+    <x:row r="426" ht="15" customHeight="1"/>
+    <x:row r="427" ht="15" customHeight="1"/>
+    <x:row r="428" ht="15" customHeight="1"/>
+    <x:row r="429" ht="15" customHeight="1"/>
+    <x:row r="430" ht="15" customHeight="1"/>
+    <x:row r="431" ht="15" customHeight="1"/>
+    <x:row r="432" ht="15" customHeight="1"/>
+    <x:row r="433" ht="15" customHeight="1"/>
+    <x:row r="434" ht="15" customHeight="1"/>
+    <x:row r="435" ht="15" customHeight="1"/>
+    <x:row r="436" ht="15" customHeight="1"/>
+    <x:row r="437" ht="15" customHeight="1"/>
+    <x:row r="438" ht="15" customHeight="1"/>
+    <x:row r="439" ht="15" customHeight="1"/>
+    <x:row r="440" ht="15" customHeight="1"/>
+    <x:row r="441" ht="15" customHeight="1"/>
+    <x:row r="442" ht="15" customHeight="1"/>
+    <x:row r="443" ht="15" customHeight="1"/>
+    <x:row r="444" ht="15" customHeight="1"/>
+    <x:row r="445" ht="15" customHeight="1"/>
+    <x:row r="446" ht="15" customHeight="1"/>
+    <x:row r="447" ht="15" customHeight="1"/>
+    <x:row r="448" ht="15" customHeight="1"/>
+    <x:row r="449" ht="15" customHeight="1"/>
+    <x:row r="450" ht="15" customHeight="1"/>
+    <x:row r="451" ht="15" customHeight="1"/>
+    <x:row r="452" ht="15" customHeight="1"/>
+    <x:row r="453" ht="15" customHeight="1"/>
+    <x:row r="454" ht="15" customHeight="1"/>
+    <x:row r="455" ht="15" customHeight="1"/>
+    <x:row r="456" ht="15" customHeight="1"/>
+    <x:row r="457" ht="15" customHeight="1"/>
+    <x:row r="458" ht="15" customHeight="1"/>
+    <x:row r="459" ht="15" customHeight="1"/>
+    <x:row r="460" ht="15" customHeight="1"/>
+    <x:row r="461" ht="15" customHeight="1"/>
+    <x:row r="462" ht="15" customHeight="1"/>
+    <x:row r="463" ht="15" customHeight="1"/>
+    <x:row r="464" ht="15" customHeight="1"/>
+    <x:row r="465" ht="15" customHeight="1"/>
+    <x:row r="466" ht="15" customHeight="1"/>
+    <x:row r="467" ht="15" customHeight="1"/>
+    <x:row r="468" ht="15" customHeight="1"/>
+    <x:row r="469" ht="15" customHeight="1"/>
+    <x:row r="470" ht="15" customHeight="1"/>
+    <x:row r="471" ht="15" customHeight="1"/>
+    <x:row r="472" ht="15" customHeight="1"/>
+    <x:row r="473" ht="15" customHeight="1"/>
+    <x:row r="474" ht="15" customHeight="1"/>
+    <x:row r="475" ht="15" customHeight="1"/>
+    <x:row r="476" ht="15" customHeight="1"/>
+    <x:row r="477" ht="15" customHeight="1"/>
+    <x:row r="478" ht="15" customHeight="1"/>
+    <x:row r="479" ht="15" customHeight="1"/>
+    <x:row r="480" ht="15" customHeight="1"/>
+    <x:row r="481" ht="15" customHeight="1"/>
+    <x:row r="482" ht="15" customHeight="1"/>
+    <x:row r="483" ht="15" customHeight="1"/>
+    <x:row r="484" ht="15" customHeight="1"/>
+    <x:row r="485" ht="15" customHeight="1"/>
+    <x:row r="486" ht="15" customHeight="1"/>
+    <x:row r="487" ht="15" customHeight="1"/>
+    <x:row r="488" ht="15" customHeight="1"/>
+    <x:row r="489" ht="15" customHeight="1"/>
+    <x:row r="490" ht="15" customHeight="1"/>
+    <x:row r="491" ht="15" customHeight="1"/>
+    <x:row r="492" ht="15" customHeight="1"/>
+    <x:row r="493" ht="15" customHeight="1"/>
+    <x:row r="494" ht="15" customHeight="1"/>
+    <x:row r="495" ht="15" customHeight="1"/>
+    <x:row r="496" ht="15" customHeight="1"/>
+    <x:row r="497" ht="15" customHeight="1"/>
+    <x:row r="498" ht="15" customHeight="1"/>
+    <x:row r="499" ht="15" customHeight="1"/>
+    <x:row r="500" ht="15" customHeight="1"/>
   </x:sheetData>
+  <x:conditionalFormatting sqref="A2:K500">
+    <x:cfRule type="expression" dxfId="11" priority="1">
+      <x:formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=0)</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="12" priority="2">
+      <x:formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=1)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4c8eb9bea614051"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R312756fb74b54147"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Restore publication metadata table styling
</commit_message>
<xml_diff>
--- a/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
+++ b/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R5bd02afd9028415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="Rfb6e92ca843a47dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R85cf037a7a29493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Topics" sheetId="2" r:id="R257ccb1108584704"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,7 +32,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -49,11 +49,6 @@
         <x:fgColor rgb="FF0B1F33"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFB4E6A2"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -62,7 +57,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -156,21 +151,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normale" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="13">
+  <x:dxfs count="11">
     <x:dxf/>
     <x:dxf/>
     <x:dxf/>
@@ -182,40 +168,25 @@
     <x:dxf/>
     <x:dxf/>
     <x:dxf/>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFB4E6A2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFD9F2D0"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:I29" totalsRowShown="0" dataDxfId="9">
-  <x:autoFilter ref="A1:I29"/>
-  <x:sortState ref="A2:I28">
-    <x:sortCondition ref="F1:F28"/>
-  </x:sortState>
-  <x:tableColumns count="9">
-    <x:tableColumn id="1" name="Title" dataDxfId="8"/>
-    <x:tableColumn id="2" name="Authors" dataDxfId="7"/>
-    <x:tableColumn id="3" name="Venue" dataDxfId="6"/>
-    <x:tableColumn id="8" name="Venue Acronym" dataDxfId="5"/>
-    <x:tableColumn id="10" name="Type" dataDxfId="4"/>
-    <x:tableColumn id="7" name="Year" dataDxfId="3"/>
-    <x:tableColumn id="5" name="Link" dataDxfId="2"/>
-    <x:tableColumn id="4" name="Bibtex" dataDxfId="1"/>
-    <x:tableColumn id="6" name="Abstract" dataDxfId="0"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K29"/>
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Title"/>
+    <x:tableColumn id="2" name="Authors"/>
+    <x:tableColumn id="3" name="Venue"/>
+    <x:tableColumn id="4" name="Venue Acronym"/>
+    <x:tableColumn id="5" name="Type"/>
+    <x:tableColumn id="6" name="Year"/>
+    <x:tableColumn id="7" name="Link"/>
+    <x:tableColumn id="8" name="Bibtex"/>
+    <x:tableColumn id="9" name="Abstract"/>
+    <x:tableColumn id="10" name="Research Topic"/>
+    <x:tableColumn id="11" name="Topic Key"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -432,37 +403,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
-      <x:c r="A1" s="35" t="str">
+      <x:c r="A1" s="18" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="B1" s="35" t="str">
+      <x:c r="B1" s="18" t="str">
         <x:v>Authors</x:v>
       </x:c>
-      <x:c r="C1" s="35" t="str">
+      <x:c r="C1" s="18" t="str">
         <x:v>Venue</x:v>
       </x:c>
-      <x:c r="D1" s="35" t="str">
+      <x:c r="D1" s="18" t="str">
         <x:v>Venue Acronym</x:v>
       </x:c>
-      <x:c r="E1" s="35" t="str">
+      <x:c r="E1" s="18" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="35" t="str">
+      <x:c r="F1" s="18" t="str">
         <x:v>Year</x:v>
       </x:c>
-      <x:c r="G1" s="35" t="str">
+      <x:c r="G1" s="18" t="str">
         <x:v>Link</x:v>
       </x:c>
-      <x:c r="H1" s="35" t="str">
+      <x:c r="H1" s="18" t="str">
         <x:v>Bibtex</x:v>
       </x:c>
-      <x:c r="I1" s="35" t="str">
+      <x:c r="I1" s="18" t="str">
         <x:v>Abstract</x:v>
       </x:c>
-      <x:c r="J1" s="35" t="str">
+      <x:c r="J1" s="18" t="str">
         <x:v>Research Topic</x:v>
       </x:c>
-      <x:c r="K1" s="35" t="str">
+      <x:c r="K1" s="18" t="str">
         <x:v>Topic Key</x:v>
       </x:c>
     </x:row>
@@ -1307,56 +1278,27 @@
     </x:row>
     <x:row r="22" ht="15" customHeight="1">
       <x:c r="A22" s="28" t="str">
-        <x:v>Memory-Augmented Prompt Tuning for Self-Supervised Continual Learning in Medical Imaging</x:v>
+        <x:v>Timely Predicting Power Mosfet Failure in EV: AI Based Metodology and Deployment at the Edge</x:v>
       </x:c>
       <x:c r="B22" s="28" t="str">
-        <x:v>-</x:v>
+        <x:v>Robin Faro, Francesco Cancelliere, Alesssandro Strano, Raffaele Mineo</x:v>
       </x:c>
       <x:c r="C22" s="28" t="str">
-        <x:v>International Workshop on Personalized Incremental Learning in Medicine (PILM)</x:v>
+        <x:v>2025 IEEE Symposia on Computational Intelligence for Energy, Transport and Environmental Sustainability (CIETES Companion)</x:v>
       </x:c>
       <x:c r="D22" s="28" t="str">
-        <x:v>PILM</x:v>
+        <x:v>CIETES Companion</x:v>
       </x:c>
       <x:c r="E22" s="28" t="str">
-        <x:v>Workshop</x:v>
+        <x:v>Conference</x:v>
       </x:c>
       <x:c r="F22" s="28" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G22" s="28"/>
-      <x:c r="H22" s="28"/>
-      <x:c r="I22" s="28"/>
-      <x:c r="J22" s="29" t="str">
-        <x:v>Adaptive, Efficient and Edge AI</x:v>
-      </x:c>
-      <x:c r="K22" s="29" t="str">
-        <x:v>efficient</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15" customHeight="1">
-      <x:c r="A23" s="28" t="str">
-        <x:v>Timely Predicting Power Mosfet Failure in EV: AI Based Metodology and Deployment at the Edge</x:v>
-      </x:c>
-      <x:c r="B23" s="28" t="str">
-        <x:v>Robin Faro, Francesco Cancelliere, Alesssandro Strano, Raffaele Mineo</x:v>
-      </x:c>
-      <x:c r="C23" s="28" t="str">
-        <x:v>2025 IEEE Symposia on Computational Intelligence for Energy, Transport and Environmental Sustainability (CIETES Companion)</x:v>
-      </x:c>
-      <x:c r="D23" s="28" t="str">
-        <x:v>CIETES Companion</x:v>
-      </x:c>
-      <x:c r="E23" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F23" s="28" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="G23" s="29" t="str">
+      <x:c r="G22" s="28" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/11003330/</x:v>
       </x:c>
-      <x:c r="H23" s="28" t="str">
+      <x:c r="H22" s="28" t="str">
         <x:v>@inproceedings{faro2025timely,
   title={Timely Predicting Power Mosfet Failure in EV: AI Based Metodology and Deployment at the Edge},
   author={Faro, Robin and Cancelliere, Francesco and Strano, Alesssandro and Mineo, Raffaele},
@@ -1366,39 +1308,39 @@
   organization={IEEE}
 }</x:v>
       </x:c>
-      <x:c r="I23" s="28" t="str">
+      <x:c r="I22" s="28" t="str">
         <x:v>Predicting the residual useful life (RUL) of power MOSFETs in electric vehicles (EVs) is crucial due to their role in transferring power from batteries to the engine. Despite its practical importance, most solutions are theoretical. This paper proposes a methodology for MOSFET RUL prediction tailored for edge devices like Nvidia Jetson ORIN and STM32. Two machine learning-based models are introduced. The first identifies the Rds(on) degradation law from a dataset that best matches the observed degradation, suitable for low-noise scenarios but lacking fine-tuning. The second model, using an autoencoder with dual decoders, is more robust. One decoder ensures the Rds(on) degradation reflects normal device behavior, while the other provides timely warnings as Rds(on) approaches critical limits, enabling proactive replacement. The paper validates these methods with theoretical and experimental datasets, emphasizing the second model's successful implementation on edge devices, demonstrating its practicality for EV applications.</x:v>
       </x:c>
-      <x:c r="J23" s="29" t="str">
+      <x:c r="J22" s="29" t="str">
         <x:v>Adaptive, Efficient and Edge AI</x:v>
       </x:c>
-      <x:c r="K23" s="29" t="str">
+      <x:c r="K22" s="29" t="str">
         <x:v>efficient</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="15" customHeight="1">
-      <x:c r="A24" s="28" t="str">
+    <x:row r="23" ht="15" customHeight="1">
+      <x:c r="A23" s="28" t="str">
         <x:v>When a model is not Enough: A Complementary AI Pipeline for Ultra-Safe PCBA Defect Detection</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="str">
+      <x:c r="B23" s="28" t="str">
         <x:v>Alberto Faro, Francesco Cancelliere, Robin Faro, Raffaele Mineo</x:v>
       </x:c>
-      <x:c r="C24" s="28" t="str">
+      <x:c r="C23" s="28" t="str">
         <x:v>The Autonomous Edge - Intelligence Embedded in Industrial Applications</x:v>
       </x:c>
-      <x:c r="D24" s="28" t="str">
+      <x:c r="D23" s="28" t="str">
         <x:v>EEAI 2025</x:v>
       </x:c>
-      <x:c r="E24" s="28" t="str">
+      <x:c r="E23" s="28" t="str">
         <x:v>Book Chapter</x:v>
       </x:c>
-      <x:c r="F24" s="28" t="n">
+      <x:c r="F23" s="28" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="G24" s="28" t="str">
+      <x:c r="G23" s="29" t="str">
         <x:v>https://www.riverpublishers.com/research_details.php?book_id=1549</x:v>
       </x:c>
-      <x:c r="H24" s="28" t="str">
+      <x:c r="H23" s="28" t="str">
         <x:v>@incollection{faro2026when,
   title={When a model is not Enough: A Complementary AI Pipeline for Ultra-Safe PCBA Defect Detection},
   author={Faro, Alberto and Cancelliere, Francesco and Faro, Robin and Mineo, Raffaele},
@@ -1410,39 +1352,39 @@
   isbn={9788743815266}
 }</x:v>
       </x:c>
-      <x:c r="I24" s="28" t="str">
+      <x:c r="I23" s="28" t="str">
         <x:v>A multi-stage automated optical inspection pipeline for safety-critical PCBA defect detection. The approach combines a transformer optimized for high recall with specialized autoencoders that reduce false positives and residual false negatives, targeting fewer than 10 false negatives per million inspected units under a high-confidence reliability requirement. The work originates from EEAI 2025 and was published as Chapter 8 of the 2026 River Publishers volume.</x:v>
       </x:c>
-      <x:c r="J24" s="29" t="str">
+      <x:c r="J23" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K24" s="29" t="str">
+      <x:c r="K23" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15" customHeight="1">
-      <x:c r="A25" s="28" t="str">
+    <x:row r="24" ht="15" customHeight="1">
+      <x:c r="A24" s="28" t="str">
         <x:v>PCB-SAID: A Low-Cost Camera-Based Dataset for Few-Shot SMD Assembly Inspection</x:v>
       </x:c>
-      <x:c r="B25" s="28" t="str">
+      <x:c r="B24" s="28" t="str">
         <x:v>Raffaele Mineo, Amelia Sorrenti, Robin Faro, Gabriele Mineo, Francesco Cancelliere, Alberto Faro</x:v>
       </x:c>
-      <x:c r="C25" s="28" t="str">
+      <x:c r="C24" s="28" t="str">
         <x:v>Proceedings of the IEEE/CVF International Conference on Computer Vision</x:v>
       </x:c>
-      <x:c r="D25" s="28" t="str">
+      <x:c r="D24" s="28" t="str">
         <x:v>ICCV</x:v>
       </x:c>
-      <x:c r="E25" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F25" s="28" t="n">
+      <x:c r="E24" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F24" s="28" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G25" s="28" t="str">
+      <x:c r="G24" s="28" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025W/VISION%2725/html/Mineo_PCB-SAID_A_Low-Cost_Camera-Based_Dataset_for_Few-Shot_SMD_Assembly_Inspection_ICCVW_2025_paper.html</x:v>
       </x:c>
-      <x:c r="H25" s="28" t="str">
+      <x:c r="H24" s="28" t="str">
         <x:v>@inproceedings{mineo2025pcb,
   title={PCB-SAID: A Low-Cost Camera-Based Dataset for Few-Shot SMD Assembly Inspection},
   author={Mineo, Raffaele and Sorrenti, Amelia and Faro, Robin and Mineo, Gabriele and Cancelliere, Francesco and Faro, Alberto},
@@ -1451,39 +1393,39 @@
   year={2025}
 }</x:v>
       </x:c>
-      <x:c r="I25" s="28" t="str">
+      <x:c r="I24" s="28" t="str">
         <x:v>Automated Optical Inspection (AOI) of surface-mounted device (SMD) assemblies is critical for ensuring quality and yield in electronics manufacturing, yet current systems rely on expensive hardware and handcrafted algorithms that struggle with novel layouts and rare defect modes. We present PCB-SAID (Printed Circuit Board – SMD Assembly Inspection Dataset), the first open, few-shot SMD inspection dataset comprising 175 RGB images annotated with 66 fine-grained classes, spanning well-soldered, mis-soldered (misaligned, lifted, rotated), missing, and short-circuit conditions, using a rigorous two-stage expert pipeline (bounding-box localization followed by polygonal mask refinement). We evaluate five state-of-the-art architectures (Fast R-CNN, DETR, YOLOv11, YOLOv12, SAM) under both full-data and few-shot (1, 5 shots) regimes, reporting mAP@[.50:.95], mAP@.50, precision, and recall. Our results reveal optimal performance gaps on rare and subtle anomalies, underscoring challenges in class imbalance and domain shift. The dataset will be made publicly available upon request to support further research in this area.</x:v>
       </x:c>
-      <x:c r="J25" s="29" t="str">
+      <x:c r="J24" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K25" s="29" t="str">
+      <x:c r="K24" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15" customHeight="1">
-      <x:c r="A26" s="28" t="str">
+    <x:row r="25" ht="15" customHeight="1">
+      <x:c r="A25" s="28" t="str">
         <x:v>BioTrak: A Blockchain-based Platform for Food Chain Logistics Traceability</x:v>
       </x:c>
-      <x:c r="B26" s="28" t="str">
+      <x:c r="B25" s="28" t="str">
         <x:v>Alessia Spitalleri, Isaak Kavasidis, Vincenzo Cartelli, Raffaele Mineo, Francesco Rundo, Simone Palazzo, Concetto Spampinato, Daniela Giordano</x:v>
       </x:c>
-      <x:c r="C26" s="28" t="str">
+      <x:c r="C25" s="28" t="str">
         <x:v>2023 International Conference on Intelligent Computing, Communication, Networking and Services (ICCNS)</x:v>
       </x:c>
-      <x:c r="D26" s="28" t="str">
+      <x:c r="D25" s="28" t="str">
         <x:v>ICCNS</x:v>
       </x:c>
-      <x:c r="E26" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F26" s="28" t="n">
+      <x:c r="E25" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F25" s="28" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G26" s="28" t="str">
+      <x:c r="G25" s="28" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10193341</x:v>
       </x:c>
-      <x:c r="H26" s="28" t="str">
+      <x:c r="H25" s="28" t="str">
         <x:v>@inproceedings{spitalleri2023biotrak,
   title={BioTrak: A blockchain-based platform for food chain logistics traceability},
   author={Spitalleri, Alessia and Kavasidis, Isaak and Cartelli, Vincenzo and Mineo, Raffaele and Rundo, Francesco and Palazzo, Simone and Spampinato, Concetto and Giordano, Daniela},
@@ -1493,39 +1435,39 @@
   organization={IEEE}
 }</x:v>
       </x:c>
-      <x:c r="I26" s="28" t="str">
+      <x:c r="I25" s="28" t="str">
         <x:v>The food supply chain, following its globalization, has become very complex. Such complexities, introduce factors that influence adversely the quality of intermediate and final products. Strict constraints regarding parameters such as maintenance temperatures and transportation times must be respected in order to ensure top quality and reduce to a minimum the detrimental effects to public health. This is a multi-factorial endeavor and all of the involved stakeholders must accept and manage the logistics burden to achieve the best possible results.However, such burden comes together with additional complexities and costs regarding data storage, business process management and company specific standard operating procedures and as such, automated methods must be devised to reduce the impact of such intrusive operations.For the above reasons, in this paper we present BioTrak: a platform capable of registering and visualizing the whole chain of transformation and transportation processes including the monitoring of cold chain logistics of food ingredients starting from the raw material producers until the final product arrives to the end-consumer.The platform includes Business Process Modelling methods to aid food supply chain stakeholders to optimize their processes and also integrates a blockchain for guaranteeing the integrity, transparency and accountability of the data.</x:v>
       </x:c>
-      <x:c r="J26" s="29" t="str">
+      <x:c r="J25" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K26" s="29" t="str">
+      <x:c r="K25" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15" customHeight="1">
-      <x:c r="A27" s="28" t="str">
+    <x:row r="26" ht="15" customHeight="1">
+      <x:c r="A26" s="28" t="str">
         <x:v>EUROVOLC - Deliverable Report - D9.3 Machine learning tool kit and database</x:v>
       </x:c>
-      <x:c r="B27" s="28" t="str">
+      <x:c r="B26" s="28" t="str">
         <x:v>S. Palazzo, R. Mineo, C. Spampinato, F. Cannavò, A. Cannata, C. Montagna, J. M. Saurel, O. Geber, A. Lemarchand</x:v>
       </x:c>
-      <x:c r="C27" s="28" t="str">
+      <x:c r="C26" s="28" t="str">
         <x:v>HORIZON 2020 EUROVOLC Project</x:v>
       </x:c>
-      <x:c r="D27" s="28" t="str">
+      <x:c r="D26" s="28" t="str">
         <x:v>EUROVOLC</x:v>
       </x:c>
-      <x:c r="E27" s="28" t="str">
+      <x:c r="E26" s="28" t="str">
         <x:v>Project</x:v>
       </x:c>
-      <x:c r="F27" s="28" t="n">
+      <x:c r="F26" s="28" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G27" s="28" t="str">
+      <x:c r="G26" s="28" t="str">
         <x:v>https://eurovolc.eu/wp-content/uploads/2021/08/D9.3.pdf</x:v>
       </x:c>
-      <x:c r="H27" s="28" t="str">
+      <x:c r="H26" s="28" t="str">
         <x:v>@techreport{palazzo2021eurovolc_d93,
   title={Machine learning tool kit and database},
   author={Palazzo, Simone and Mineo, Raffaele and Spampinato, Concetto and Cannav{\`o}, Flavio and Cannata, Andrea and Montagna, Chiara and Saurel, Jean-Marie and Geber, O. and Lemarchand, Arnaud},
@@ -1535,39 +1477,39 @@
   note={Horizon 2020 {EUROVOLC}, Grant Agreement No. 731070}
 }</x:v>
       </x:c>
-      <x:c r="I27" s="28" t="str">
+      <x:c r="I26" s="28" t="str">
         <x:v>The recent success of deep learning techniques has stimulated the application of such approaches for the automatic identification of models related to volcanic phenomena. In this study, a tool was developed for anomaly detection in historical volcanic data in an unsupervised manner. The results on data from Etna and Stromboli are promising, highlighting the ability to anticipate significant anomalies with respect to volcanic events.</x:v>
       </x:c>
-      <x:c r="J27" s="29" t="str">
+      <x:c r="J26" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K27" s="29" t="str">
+      <x:c r="K26" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" customHeight="1">
-      <x:c r="A28" s="28" t="str">
+    <x:row r="27" ht="15" customHeight="1">
+      <x:c r="A27" s="28" t="str">
         <x:v>VOLcano UNrest Detection (VolUnD) Toolkit</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="str">
+      <x:c r="B27" s="28" t="str">
         <x:v>R. Mineo, P. Spadaro, F. Cannavò, S. Palazzo, A. Cannata, C. Spampinato</x:v>
       </x:c>
-      <x:c r="C28" s="28" t="str">
+      <x:c r="C27" s="28" t="str">
         <x:v>Zenodo</x:v>
       </x:c>
-      <x:c r="D28" s="28" t="str">
+      <x:c r="D27" s="28" t="str">
         <x:v>Zenodo</x:v>
       </x:c>
-      <x:c r="E28" s="28" t="str">
+      <x:c r="E27" s="28" t="str">
         <x:v>Software</x:v>
       </x:c>
-      <x:c r="F28" s="28" t="n">
+      <x:c r="F27" s="28" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G28" s="30" t="str">
+      <x:c r="G27" s="28" t="str">
         <x:v>https://zenodo.org/records/5541125</x:v>
       </x:c>
-      <x:c r="H28" s="30" t="str">
+      <x:c r="H27" s="28" t="str">
         <x:v>@misc{raffaele_mineo_2021_5541125,
   title={EUROVOLC-ML/VolUnD-Toolkit: VolUnD v1.0},
   author={Mineo, Raffaele and Spadaro, Paolo and Cannav{\`o}, Flavio and Palazzo, Simone and Cannata, Andrea and Spampinato, Concetto},
@@ -1576,39 +1518,39 @@
   doi={10.5281/zenodo.5541125}
 }</x:v>
       </x:c>
-      <x:c r="I28" s="28" t="str">
+      <x:c r="I27" s="28" t="str">
         <x:v>VolUnD is a VOLcano UNrest Detection toolkit written in (PyTorch) Python. Performs anomaly detection of historical volcanic data in an unsupervised manner, leveraging the hypothesis that normal activity dominates the distribution of events and can therefore be treated as the main source of information for training a model capable of identifying deviations as anomalies. These anomalies could be attributed to changes in the state of the volcano.</x:v>
       </x:c>
-      <x:c r="J28" s="29" t="str">
+      <x:c r="J27" s="29" t="str">
         <x:v>Scientific and Industrial Intelligent Systems</x:v>
       </x:c>
-      <x:c r="K28" s="29" t="str">
+      <x:c r="K27" s="29" t="str">
         <x:v>scientific</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="15" customHeight="1">
-      <x:c r="A29" s="28" t="str">
+    <x:row r="28" ht="15" customHeight="1">
+      <x:c r="A28" s="28" t="str">
         <x:v>Advancing Healthcare with Multimodal AI: Enhanced Diagnosis, Cognitive Monitoring, and Inclusive Medical Communication</x:v>
       </x:c>
-      <x:c r="B29" s="28" t="str">
+      <x:c r="B28" s="28" t="str">
         <x:v>Raffaele Mineo</x:v>
       </x:c>
-      <x:c r="C29" s="28" t="str">
+      <x:c r="C28" s="28" t="str">
         <x:v>International Conference on Medical Image Computing and Computer-Assisted Intervention</x:v>
       </x:c>
-      <x:c r="D29" s="28" t="str">
+      <x:c r="D28" s="28" t="str">
         <x:v>MICCAI</x:v>
       </x:c>
-      <x:c r="E29" s="28" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="F29" s="28" t="n">
+      <x:c r="E28" s="28" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="F28" s="28" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="G29" s="28" t="str">
+      <x:c r="G28" s="30" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="H29" s="28" t="str">
+      <x:c r="H28" s="30" t="str">
         <x:v>@inproceedings{mineo2025advancing,
   title={Advancing Healthcare with Multimodal AI: Enhanced Diagnosis, Cognitive Monitoring, and Inclusive Medical Communication},
   author={Mineo, Raffaele},
@@ -1617,39 +1559,39 @@
   organization={Springer}
 }</x:v>
       </x:c>
-      <x:c r="I29" s="28" t="str">
+      <x:c r="I28" s="28" t="str">
         <x:v>This doctoral research explores multimodal deep learning to enhance diagnosis, cognitive monitoring, and communication accessibility in healthcare. Across three clinical domains - cardiovascular diagnostics, neurocognitive assessment, and sign language recognition - we develop transformer-based pipelines tailored for real-time applicability, interpretability, and privacy compliance. In the cardiovascular setting, we propose spatio-temporal models for non-invasive estimation of FFR and iFR from single-view coronary angiography, integrating convolutional and transformer encoders with multi-task supervision. These innovations culminate in the STARFLOW system, a deployable platform achieving high accuracy in multicenter studies, and protected by national and EU patents. For cognitive screening, we introduce pipelines that analyze facial micro-movements and eye-gaze trajectories using phase-based motion magnification, attention-based encoders, and a novel Time-Aware Positional Embedding (TAPE) module. These systems enable automated scoring of MMSE and MoCA using commodity tablets, facilitating contactless and scalable cognitive health tools. To promote inclusivity, we release MultiMedaLIS, the first multimodal dataset of Italian medical sign language, and develop a GDPR-compliant radar-based recognition pipeline using Range-Doppler Maps and temporal transformers. This system ensures robust gesture classification under privacy and environmental constraints. Collectively, this work contributes a unified framework for interpretable and adaptive AI in healthcare, advancing real-world integration through methodological innovation, validated deployment, and alignment with clinical needs.</x:v>
       </x:c>
-      <x:c r="J29" s="29" t="str">
+      <x:c r="J28" s="29" t="str">
         <x:v>Research Synthesis and Scholarly Outputs</x:v>
       </x:c>
-      <x:c r="K29" s="29" t="str">
+      <x:c r="K28" s="29" t="str">
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="15" customHeight="1">
-      <x:c r="A30" s="37" t="str">
+    <x:row r="29" ht="15" customHeight="1">
+      <x:c r="A29" s="28" t="str">
         <x:v>Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25)</x:v>
       </x:c>
-      <x:c r="B30" s="37" t="str">
+      <x:c r="B29" s="28" t="str">
         <x:v>Simone Palazzo, Giovanni Bellitto, Raffaele Mineo, Amelia Sorrenti, Camila Gonzalez, Angelo Porrello, Lorenzo Bonicelli</x:v>
       </x:c>
-      <x:c r="C30" s="37" t="str">
+      <x:c r="C29" s="28" t="str">
         <x:v>ACM Multimedia 2025</x:v>
       </x:c>
-      <x:c r="D30" s="37" t="str">
+      <x:c r="D29" s="28" t="str">
         <x:v>ACM MM</x:v>
       </x:c>
-      <x:c r="E30" s="37" t="str">
+      <x:c r="E29" s="28" t="str">
         <x:v>Edited Proceedings</x:v>
       </x:c>
-      <x:c r="F30" s="37" t="n">
+      <x:c r="F29" s="28" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="G30" s="37" t="str">
+      <x:c r="G29" s="28" t="str">
         <x:v>https://dl.acm.org/doi/pdf/10.1145/3746259</x:v>
       </x:c>
-      <x:c r="H30" s="37" t="str">
+      <x:c r="H29" s="28" t="str">
         <x:v>@proceedings{pilm2025,
   title={Proceedings of the International Workshop on Personalized Incremental Learning in Medicine (PILM ’25), co-located with ACM Multimedia 2025},
   editor={Palazzo, Simone and Bellitto, Giovanni and Mineo, Raffaele and Sorrenti, Amelia and Gonzalez, Camila and Porrello, Angelo and Bonicelli, Lorenzo},
@@ -1658,498 +1600,33 @@
   doi={10.1145/3746259}
 }</x:v>
       </x:c>
-      <x:c r="I30" s="37" t="str">
+      <x:c r="I29" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="J30" s="38" t="str">
+      <x:c r="J29" s="29" t="str">
         <x:v>Research Synthesis and Scholarly Outputs</x:v>
       </x:c>
-      <x:c r="K30" s="38" t="str">
+      <x:c r="K29" s="29" t="str">
         <x:v>synthesis</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="15" customHeight="1"/>
-    <x:row r="32" ht="15" customHeight="1"/>
-    <x:row r="33" ht="15" customHeight="1"/>
-    <x:row r="34" ht="15" customHeight="1"/>
-    <x:row r="35" ht="15" customHeight="1"/>
-    <x:row r="36" ht="15" customHeight="1"/>
-    <x:row r="37" ht="15" customHeight="1"/>
-    <x:row r="38" ht="15" customHeight="1"/>
-    <x:row r="39" ht="15" customHeight="1"/>
-    <x:row r="40" ht="15" customHeight="1"/>
-    <x:row r="41" ht="15" customHeight="1"/>
-    <x:row r="42" ht="15" customHeight="1"/>
-    <x:row r="43" ht="15" customHeight="1"/>
-    <x:row r="44" ht="15" customHeight="1"/>
-    <x:row r="45" ht="15" customHeight="1"/>
-    <x:row r="46" ht="15" customHeight="1"/>
-    <x:row r="47" ht="15" customHeight="1"/>
-    <x:row r="48" ht="15" customHeight="1"/>
-    <x:row r="49" ht="15" customHeight="1"/>
-    <x:row r="50" ht="15" customHeight="1"/>
-    <x:row r="51" ht="15" customHeight="1"/>
-    <x:row r="52" ht="15" customHeight="1"/>
-    <x:row r="53" ht="15" customHeight="1"/>
-    <x:row r="54" ht="15" customHeight="1"/>
-    <x:row r="55" ht="15" customHeight="1"/>
-    <x:row r="56" ht="15" customHeight="1"/>
-    <x:row r="57" ht="15" customHeight="1"/>
-    <x:row r="58" ht="15" customHeight="1"/>
-    <x:row r="59" ht="15" customHeight="1"/>
-    <x:row r="60" ht="15" customHeight="1"/>
-    <x:row r="61" ht="15" customHeight="1"/>
-    <x:row r="62" ht="15" customHeight="1"/>
-    <x:row r="63" ht="15" customHeight="1"/>
-    <x:row r="64" ht="15" customHeight="1"/>
-    <x:row r="65" ht="15" customHeight="1"/>
-    <x:row r="66" ht="15" customHeight="1"/>
-    <x:row r="67" ht="15" customHeight="1"/>
-    <x:row r="68" ht="15" customHeight="1"/>
-    <x:row r="69" ht="15" customHeight="1"/>
-    <x:row r="70" ht="15" customHeight="1"/>
-    <x:row r="71" ht="15" customHeight="1"/>
-    <x:row r="72" ht="15" customHeight="1"/>
-    <x:row r="73" ht="15" customHeight="1"/>
-    <x:row r="74" ht="15" customHeight="1"/>
-    <x:row r="75" ht="15" customHeight="1"/>
-    <x:row r="76" ht="15" customHeight="1"/>
-    <x:row r="77" ht="15" customHeight="1"/>
-    <x:row r="78" ht="15" customHeight="1"/>
-    <x:row r="79" ht="15" customHeight="1"/>
-    <x:row r="80" ht="15" customHeight="1"/>
-    <x:row r="81" ht="15" customHeight="1"/>
-    <x:row r="82" ht="15" customHeight="1"/>
-    <x:row r="83" ht="15" customHeight="1"/>
-    <x:row r="84" ht="15" customHeight="1"/>
-    <x:row r="85" ht="15" customHeight="1"/>
-    <x:row r="86" ht="15" customHeight="1"/>
-    <x:row r="87" ht="15" customHeight="1"/>
-    <x:row r="88" ht="15" customHeight="1"/>
-    <x:row r="89" ht="15" customHeight="1"/>
-    <x:row r="90" ht="15" customHeight="1"/>
-    <x:row r="91" ht="15" customHeight="1"/>
-    <x:row r="92" ht="15" customHeight="1"/>
-    <x:row r="93" ht="15" customHeight="1"/>
-    <x:row r="94" ht="15" customHeight="1"/>
-    <x:row r="95" ht="15" customHeight="1"/>
-    <x:row r="96" ht="15" customHeight="1"/>
-    <x:row r="97" ht="15" customHeight="1"/>
-    <x:row r="98" ht="15" customHeight="1"/>
-    <x:row r="99" ht="15" customHeight="1"/>
-    <x:row r="100" ht="15" customHeight="1"/>
-    <x:row r="101" ht="15" customHeight="1"/>
-    <x:row r="102" ht="15" customHeight="1"/>
-    <x:row r="103" ht="15" customHeight="1"/>
-    <x:row r="104" ht="15" customHeight="1"/>
-    <x:row r="105" ht="15" customHeight="1"/>
-    <x:row r="106" ht="15" customHeight="1"/>
-    <x:row r="107" ht="15" customHeight="1"/>
-    <x:row r="108" ht="15" customHeight="1"/>
-    <x:row r="109" ht="15" customHeight="1"/>
-    <x:row r="110" ht="15" customHeight="1"/>
-    <x:row r="111" ht="15" customHeight="1"/>
-    <x:row r="112" ht="15" customHeight="1"/>
-    <x:row r="113" ht="15" customHeight="1"/>
-    <x:row r="114" ht="15" customHeight="1"/>
-    <x:row r="115" ht="15" customHeight="1"/>
-    <x:row r="116" ht="15" customHeight="1"/>
-    <x:row r="117" ht="15" customHeight="1"/>
-    <x:row r="118" ht="15" customHeight="1"/>
-    <x:row r="119" ht="15" customHeight="1"/>
-    <x:row r="120" ht="15" customHeight="1"/>
-    <x:row r="121" ht="15" customHeight="1"/>
-    <x:row r="122" ht="15" customHeight="1"/>
-    <x:row r="123" ht="15" customHeight="1"/>
-    <x:row r="124" ht="15" customHeight="1"/>
-    <x:row r="125" ht="15" customHeight="1"/>
-    <x:row r="126" ht="15" customHeight="1"/>
-    <x:row r="127" ht="15" customHeight="1"/>
-    <x:row r="128" ht="15" customHeight="1"/>
-    <x:row r="129" ht="15" customHeight="1"/>
-    <x:row r="130" ht="15" customHeight="1"/>
-    <x:row r="131" ht="15" customHeight="1"/>
-    <x:row r="132" ht="15" customHeight="1"/>
-    <x:row r="133" ht="15" customHeight="1"/>
-    <x:row r="134" ht="15" customHeight="1"/>
-    <x:row r="135" ht="15" customHeight="1"/>
-    <x:row r="136" ht="15" customHeight="1"/>
-    <x:row r="137" ht="15" customHeight="1"/>
-    <x:row r="138" ht="15" customHeight="1"/>
-    <x:row r="139" ht="15" customHeight="1"/>
-    <x:row r="140" ht="15" customHeight="1"/>
-    <x:row r="141" ht="15" customHeight="1"/>
-    <x:row r="142" ht="15" customHeight="1"/>
-    <x:row r="143" ht="15" customHeight="1"/>
-    <x:row r="144" ht="15" customHeight="1"/>
-    <x:row r="145" ht="15" customHeight="1"/>
-    <x:row r="146" ht="15" customHeight="1"/>
-    <x:row r="147" ht="15" customHeight="1"/>
-    <x:row r="148" ht="15" customHeight="1"/>
-    <x:row r="149" ht="15" customHeight="1"/>
-    <x:row r="150" ht="15" customHeight="1"/>
-    <x:row r="151" ht="15" customHeight="1"/>
-    <x:row r="152" ht="15" customHeight="1"/>
-    <x:row r="153" ht="15" customHeight="1"/>
-    <x:row r="154" ht="15" customHeight="1"/>
-    <x:row r="155" ht="15" customHeight="1"/>
-    <x:row r="156" ht="15" customHeight="1"/>
-    <x:row r="157" ht="15" customHeight="1"/>
-    <x:row r="158" ht="15" customHeight="1"/>
-    <x:row r="159" ht="15" customHeight="1"/>
-    <x:row r="160" ht="15" customHeight="1"/>
-    <x:row r="161" ht="15" customHeight="1"/>
-    <x:row r="162" ht="15" customHeight="1"/>
-    <x:row r="163" ht="15" customHeight="1"/>
-    <x:row r="164" ht="15" customHeight="1"/>
-    <x:row r="165" ht="15" customHeight="1"/>
-    <x:row r="166" ht="15" customHeight="1"/>
-    <x:row r="167" ht="15" customHeight="1"/>
-    <x:row r="168" ht="15" customHeight="1"/>
-    <x:row r="169" ht="15" customHeight="1"/>
-    <x:row r="170" ht="15" customHeight="1"/>
-    <x:row r="171" ht="15" customHeight="1"/>
-    <x:row r="172" ht="15" customHeight="1"/>
-    <x:row r="173" ht="15" customHeight="1"/>
-    <x:row r="174" ht="15" customHeight="1"/>
-    <x:row r="175" ht="15" customHeight="1"/>
-    <x:row r="176" ht="15" customHeight="1"/>
-    <x:row r="177" ht="15" customHeight="1"/>
-    <x:row r="178" ht="15" customHeight="1"/>
-    <x:row r="179" ht="15" customHeight="1"/>
-    <x:row r="180" ht="15" customHeight="1"/>
-    <x:row r="181" ht="15" customHeight="1"/>
-    <x:row r="182" ht="15" customHeight="1"/>
-    <x:row r="183" ht="15" customHeight="1"/>
-    <x:row r="184" ht="15" customHeight="1"/>
-    <x:row r="185" ht="15" customHeight="1"/>
-    <x:row r="186" ht="15" customHeight="1"/>
-    <x:row r="187" ht="15" customHeight="1"/>
-    <x:row r="188" ht="15" customHeight="1"/>
-    <x:row r="189" ht="15" customHeight="1"/>
-    <x:row r="190" ht="15" customHeight="1"/>
-    <x:row r="191" ht="15" customHeight="1"/>
-    <x:row r="192" ht="15" customHeight="1"/>
-    <x:row r="193" ht="15" customHeight="1"/>
-    <x:row r="194" ht="15" customHeight="1"/>
-    <x:row r="195" ht="15" customHeight="1"/>
-    <x:row r="196" ht="15" customHeight="1"/>
-    <x:row r="197" ht="15" customHeight="1"/>
-    <x:row r="198" ht="15" customHeight="1"/>
-    <x:row r="199" ht="15" customHeight="1"/>
-    <x:row r="200" ht="15" customHeight="1"/>
-    <x:row r="201" ht="15" customHeight="1"/>
-    <x:row r="202" ht="15" customHeight="1"/>
-    <x:row r="203" ht="15" customHeight="1"/>
-    <x:row r="204" ht="15" customHeight="1"/>
-    <x:row r="205" ht="15" customHeight="1"/>
-    <x:row r="206" ht="15" customHeight="1"/>
-    <x:row r="207" ht="15" customHeight="1"/>
-    <x:row r="208" ht="15" customHeight="1"/>
-    <x:row r="209" ht="15" customHeight="1"/>
-    <x:row r="210" ht="15" customHeight="1"/>
-    <x:row r="211" ht="15" customHeight="1"/>
-    <x:row r="212" ht="15" customHeight="1"/>
-    <x:row r="213" ht="15" customHeight="1"/>
-    <x:row r="214" ht="15" customHeight="1"/>
-    <x:row r="215" ht="15" customHeight="1"/>
-    <x:row r="216" ht="15" customHeight="1"/>
-    <x:row r="217" ht="15" customHeight="1"/>
-    <x:row r="218" ht="15" customHeight="1"/>
-    <x:row r="219" ht="15" customHeight="1"/>
-    <x:row r="220" ht="15" customHeight="1"/>
-    <x:row r="221" ht="15" customHeight="1"/>
-    <x:row r="222" ht="15" customHeight="1"/>
-    <x:row r="223" ht="15" customHeight="1"/>
-    <x:row r="224" ht="15" customHeight="1"/>
-    <x:row r="225" ht="15" customHeight="1"/>
-    <x:row r="226" ht="15" customHeight="1"/>
-    <x:row r="227" ht="15" customHeight="1"/>
-    <x:row r="228" ht="15" customHeight="1"/>
-    <x:row r="229" ht="15" customHeight="1"/>
-    <x:row r="230" ht="15" customHeight="1"/>
-    <x:row r="231" ht="15" customHeight="1"/>
-    <x:row r="232" ht="15" customHeight="1"/>
-    <x:row r="233" ht="15" customHeight="1"/>
-    <x:row r="234" ht="15" customHeight="1"/>
-    <x:row r="235" ht="15" customHeight="1"/>
-    <x:row r="236" ht="15" customHeight="1"/>
-    <x:row r="237" ht="15" customHeight="1"/>
-    <x:row r="238" ht="15" customHeight="1"/>
-    <x:row r="239" ht="15" customHeight="1"/>
-    <x:row r="240" ht="15" customHeight="1"/>
-    <x:row r="241" ht="15" customHeight="1"/>
-    <x:row r="242" ht="15" customHeight="1"/>
-    <x:row r="243" ht="15" customHeight="1"/>
-    <x:row r="244" ht="15" customHeight="1"/>
-    <x:row r="245" ht="15" customHeight="1"/>
-    <x:row r="246" ht="15" customHeight="1"/>
-    <x:row r="247" ht="15" customHeight="1"/>
-    <x:row r="248" ht="15" customHeight="1"/>
-    <x:row r="249" ht="15" customHeight="1"/>
-    <x:row r="250" ht="15" customHeight="1"/>
-    <x:row r="251" ht="15" customHeight="1"/>
-    <x:row r="252" ht="15" customHeight="1"/>
-    <x:row r="253" ht="15" customHeight="1"/>
-    <x:row r="254" ht="15" customHeight="1"/>
-    <x:row r="255" ht="15" customHeight="1"/>
-    <x:row r="256" ht="15" customHeight="1"/>
-    <x:row r="257" ht="15" customHeight="1"/>
-    <x:row r="258" ht="15" customHeight="1"/>
-    <x:row r="259" ht="15" customHeight="1"/>
-    <x:row r="260" ht="15" customHeight="1"/>
-    <x:row r="261" ht="15" customHeight="1"/>
-    <x:row r="262" ht="15" customHeight="1"/>
-    <x:row r="263" ht="15" customHeight="1"/>
-    <x:row r="264" ht="15" customHeight="1"/>
-    <x:row r="265" ht="15" customHeight="1"/>
-    <x:row r="266" ht="15" customHeight="1"/>
-    <x:row r="267" ht="15" customHeight="1"/>
-    <x:row r="268" ht="15" customHeight="1"/>
-    <x:row r="269" ht="15" customHeight="1"/>
-    <x:row r="270" ht="15" customHeight="1"/>
-    <x:row r="271" ht="15" customHeight="1"/>
-    <x:row r="272" ht="15" customHeight="1"/>
-    <x:row r="273" ht="15" customHeight="1"/>
-    <x:row r="274" ht="15" customHeight="1"/>
-    <x:row r="275" ht="15" customHeight="1"/>
-    <x:row r="276" ht="15" customHeight="1"/>
-    <x:row r="277" ht="15" customHeight="1"/>
-    <x:row r="278" ht="15" customHeight="1"/>
-    <x:row r="279" ht="15" customHeight="1"/>
-    <x:row r="280" ht="15" customHeight="1"/>
-    <x:row r="281" ht="15" customHeight="1"/>
-    <x:row r="282" ht="15" customHeight="1"/>
-    <x:row r="283" ht="15" customHeight="1"/>
-    <x:row r="284" ht="15" customHeight="1"/>
-    <x:row r="285" ht="15" customHeight="1"/>
-    <x:row r="286" ht="15" customHeight="1"/>
-    <x:row r="287" ht="15" customHeight="1"/>
-    <x:row r="288" ht="15" customHeight="1"/>
-    <x:row r="289" ht="15" customHeight="1"/>
-    <x:row r="290" ht="15" customHeight="1"/>
-    <x:row r="291" ht="15" customHeight="1"/>
-    <x:row r="292" ht="15" customHeight="1"/>
-    <x:row r="293" ht="15" customHeight="1"/>
-    <x:row r="294" ht="15" customHeight="1"/>
-    <x:row r="295" ht="15" customHeight="1"/>
-    <x:row r="296" ht="15" customHeight="1"/>
-    <x:row r="297" ht="15" customHeight="1"/>
-    <x:row r="298" ht="15" customHeight="1"/>
-    <x:row r="299" ht="15" customHeight="1"/>
-    <x:row r="300" ht="15" customHeight="1"/>
-    <x:row r="301" ht="15" customHeight="1"/>
-    <x:row r="302" ht="15" customHeight="1"/>
-    <x:row r="303" ht="15" customHeight="1"/>
-    <x:row r="304" ht="15" customHeight="1"/>
-    <x:row r="305" ht="15" customHeight="1"/>
-    <x:row r="306" ht="15" customHeight="1"/>
-    <x:row r="307" ht="15" customHeight="1"/>
-    <x:row r="308" ht="15" customHeight="1"/>
-    <x:row r="309" ht="15" customHeight="1"/>
-    <x:row r="310" ht="15" customHeight="1"/>
-    <x:row r="311" ht="15" customHeight="1"/>
-    <x:row r="312" ht="15" customHeight="1"/>
-    <x:row r="313" ht="15" customHeight="1"/>
-    <x:row r="314" ht="15" customHeight="1"/>
-    <x:row r="315" ht="15" customHeight="1"/>
-    <x:row r="316" ht="15" customHeight="1"/>
-    <x:row r="317" ht="15" customHeight="1"/>
-    <x:row r="318" ht="15" customHeight="1"/>
-    <x:row r="319" ht="15" customHeight="1"/>
-    <x:row r="320" ht="15" customHeight="1"/>
-    <x:row r="321" ht="15" customHeight="1"/>
-    <x:row r="322" ht="15" customHeight="1"/>
-    <x:row r="323" ht="15" customHeight="1"/>
-    <x:row r="324" ht="15" customHeight="1"/>
-    <x:row r="325" ht="15" customHeight="1"/>
-    <x:row r="326" ht="15" customHeight="1"/>
-    <x:row r="327" ht="15" customHeight="1"/>
-    <x:row r="328" ht="15" customHeight="1"/>
-    <x:row r="329" ht="15" customHeight="1"/>
-    <x:row r="330" ht="15" customHeight="1"/>
-    <x:row r="331" ht="15" customHeight="1"/>
-    <x:row r="332" ht="15" customHeight="1"/>
-    <x:row r="333" ht="15" customHeight="1"/>
-    <x:row r="334" ht="15" customHeight="1"/>
-    <x:row r="335" ht="15" customHeight="1"/>
-    <x:row r="336" ht="15" customHeight="1"/>
-    <x:row r="337" ht="15" customHeight="1"/>
-    <x:row r="338" ht="15" customHeight="1"/>
-    <x:row r="339" ht="15" customHeight="1"/>
-    <x:row r="340" ht="15" customHeight="1"/>
-    <x:row r="341" ht="15" customHeight="1"/>
-    <x:row r="342" ht="15" customHeight="1"/>
-    <x:row r="343" ht="15" customHeight="1"/>
-    <x:row r="344" ht="15" customHeight="1"/>
-    <x:row r="345" ht="15" customHeight="1"/>
-    <x:row r="346" ht="15" customHeight="1"/>
-    <x:row r="347" ht="15" customHeight="1"/>
-    <x:row r="348" ht="15" customHeight="1"/>
-    <x:row r="349" ht="15" customHeight="1"/>
-    <x:row r="350" ht="15" customHeight="1"/>
-    <x:row r="351" ht="15" customHeight="1"/>
-    <x:row r="352" ht="15" customHeight="1"/>
-    <x:row r="353" ht="15" customHeight="1"/>
-    <x:row r="354" ht="15" customHeight="1"/>
-    <x:row r="355" ht="15" customHeight="1"/>
-    <x:row r="356" ht="15" customHeight="1"/>
-    <x:row r="357" ht="15" customHeight="1"/>
-    <x:row r="358" ht="15" customHeight="1"/>
-    <x:row r="359" ht="15" customHeight="1"/>
-    <x:row r="360" ht="15" customHeight="1"/>
-    <x:row r="361" ht="15" customHeight="1"/>
-    <x:row r="362" ht="15" customHeight="1"/>
-    <x:row r="363" ht="15" customHeight="1"/>
-    <x:row r="364" ht="15" customHeight="1"/>
-    <x:row r="365" ht="15" customHeight="1"/>
-    <x:row r="366" ht="15" customHeight="1"/>
-    <x:row r="367" ht="15" customHeight="1"/>
-    <x:row r="368" ht="15" customHeight="1"/>
-    <x:row r="369" ht="15" customHeight="1"/>
-    <x:row r="370" ht="15" customHeight="1"/>
-    <x:row r="371" ht="15" customHeight="1"/>
-    <x:row r="372" ht="15" customHeight="1"/>
-    <x:row r="373" ht="15" customHeight="1"/>
-    <x:row r="374" ht="15" customHeight="1"/>
-    <x:row r="375" ht="15" customHeight="1"/>
-    <x:row r="376" ht="15" customHeight="1"/>
-    <x:row r="377" ht="15" customHeight="1"/>
-    <x:row r="378" ht="15" customHeight="1"/>
-    <x:row r="379" ht="15" customHeight="1"/>
-    <x:row r="380" ht="15" customHeight="1"/>
-    <x:row r="381" ht="15" customHeight="1"/>
-    <x:row r="382" ht="15" customHeight="1"/>
-    <x:row r="383" ht="15" customHeight="1"/>
-    <x:row r="384" ht="15" customHeight="1"/>
-    <x:row r="385" ht="15" customHeight="1"/>
-    <x:row r="386" ht="15" customHeight="1"/>
-    <x:row r="387" ht="15" customHeight="1"/>
-    <x:row r="388" ht="15" customHeight="1"/>
-    <x:row r="389" ht="15" customHeight="1"/>
-    <x:row r="390" ht="15" customHeight="1"/>
-    <x:row r="391" ht="15" customHeight="1"/>
-    <x:row r="392" ht="15" customHeight="1"/>
-    <x:row r="393" ht="15" customHeight="1"/>
-    <x:row r="394" ht="15" customHeight="1"/>
-    <x:row r="395" ht="15" customHeight="1"/>
-    <x:row r="396" ht="15" customHeight="1"/>
-    <x:row r="397" ht="15" customHeight="1"/>
-    <x:row r="398" ht="15" customHeight="1"/>
-    <x:row r="399" ht="15" customHeight="1"/>
-    <x:row r="400" ht="15" customHeight="1"/>
-    <x:row r="401" ht="15" customHeight="1"/>
-    <x:row r="402" ht="15" customHeight="1"/>
-    <x:row r="403" ht="15" customHeight="1"/>
-    <x:row r="404" ht="15" customHeight="1"/>
-    <x:row r="405" ht="15" customHeight="1"/>
-    <x:row r="406" ht="15" customHeight="1"/>
-    <x:row r="407" ht="15" customHeight="1"/>
-    <x:row r="408" ht="15" customHeight="1"/>
-    <x:row r="409" ht="15" customHeight="1"/>
-    <x:row r="410" ht="15" customHeight="1"/>
-    <x:row r="411" ht="15" customHeight="1"/>
-    <x:row r="412" ht="15" customHeight="1"/>
-    <x:row r="413" ht="15" customHeight="1"/>
-    <x:row r="414" ht="15" customHeight="1"/>
-    <x:row r="415" ht="15" customHeight="1"/>
-    <x:row r="416" ht="15" customHeight="1"/>
-    <x:row r="417" ht="15" customHeight="1"/>
-    <x:row r="418" ht="15" customHeight="1"/>
-    <x:row r="419" ht="15" customHeight="1"/>
-    <x:row r="420" ht="15" customHeight="1"/>
-    <x:row r="421" ht="15" customHeight="1"/>
-    <x:row r="422" ht="15" customHeight="1"/>
-    <x:row r="423" ht="15" customHeight="1"/>
-    <x:row r="424" ht="15" customHeight="1"/>
-    <x:row r="425" ht="15" customHeight="1"/>
-    <x:row r="426" ht="15" customHeight="1"/>
-    <x:row r="427" ht="15" customHeight="1"/>
-    <x:row r="428" ht="15" customHeight="1"/>
-    <x:row r="429" ht="15" customHeight="1"/>
-    <x:row r="430" ht="15" customHeight="1"/>
-    <x:row r="431" ht="15" customHeight="1"/>
-    <x:row r="432" ht="15" customHeight="1"/>
-    <x:row r="433" ht="15" customHeight="1"/>
-    <x:row r="434" ht="15" customHeight="1"/>
-    <x:row r="435" ht="15" customHeight="1"/>
-    <x:row r="436" ht="15" customHeight="1"/>
-    <x:row r="437" ht="15" customHeight="1"/>
-    <x:row r="438" ht="15" customHeight="1"/>
-    <x:row r="439" ht="15" customHeight="1"/>
-    <x:row r="440" ht="15" customHeight="1"/>
-    <x:row r="441" ht="15" customHeight="1"/>
-    <x:row r="442" ht="15" customHeight="1"/>
-    <x:row r="443" ht="15" customHeight="1"/>
-    <x:row r="444" ht="15" customHeight="1"/>
-    <x:row r="445" ht="15" customHeight="1"/>
-    <x:row r="446" ht="15" customHeight="1"/>
-    <x:row r="447" ht="15" customHeight="1"/>
-    <x:row r="448" ht="15" customHeight="1"/>
-    <x:row r="449" ht="15" customHeight="1"/>
-    <x:row r="450" ht="15" customHeight="1"/>
-    <x:row r="451" ht="15" customHeight="1"/>
-    <x:row r="452" ht="15" customHeight="1"/>
-    <x:row r="453" ht="15" customHeight="1"/>
-    <x:row r="454" ht="15" customHeight="1"/>
-    <x:row r="455" ht="15" customHeight="1"/>
-    <x:row r="456" ht="15" customHeight="1"/>
-    <x:row r="457" ht="15" customHeight="1"/>
-    <x:row r="458" ht="15" customHeight="1"/>
-    <x:row r="459" ht="15" customHeight="1"/>
-    <x:row r="460" ht="15" customHeight="1"/>
-    <x:row r="461" ht="15" customHeight="1"/>
-    <x:row r="462" ht="15" customHeight="1"/>
-    <x:row r="463" ht="15" customHeight="1"/>
-    <x:row r="464" ht="15" customHeight="1"/>
-    <x:row r="465" ht="15" customHeight="1"/>
-    <x:row r="466" ht="15" customHeight="1"/>
-    <x:row r="467" ht="15" customHeight="1"/>
-    <x:row r="468" ht="15" customHeight="1"/>
-    <x:row r="469" ht="15" customHeight="1"/>
-    <x:row r="470" ht="15" customHeight="1"/>
-    <x:row r="471" ht="15" customHeight="1"/>
-    <x:row r="472" ht="15" customHeight="1"/>
-    <x:row r="473" ht="15" customHeight="1"/>
-    <x:row r="474" ht="15" customHeight="1"/>
-    <x:row r="475" ht="15" customHeight="1"/>
-    <x:row r="476" ht="15" customHeight="1"/>
-    <x:row r="477" ht="15" customHeight="1"/>
-    <x:row r="478" ht="15" customHeight="1"/>
-    <x:row r="479" ht="15" customHeight="1"/>
-    <x:row r="480" ht="15" customHeight="1"/>
-    <x:row r="481" ht="15" customHeight="1"/>
-    <x:row r="482" ht="15" customHeight="1"/>
-    <x:row r="483" ht="15" customHeight="1"/>
-    <x:row r="484" ht="15" customHeight="1"/>
-    <x:row r="485" ht="15" customHeight="1"/>
-    <x:row r="486" ht="15" customHeight="1"/>
-    <x:row r="487" ht="15" customHeight="1"/>
-    <x:row r="488" ht="15" customHeight="1"/>
-    <x:row r="489" ht="15" customHeight="1"/>
-    <x:row r="490" ht="15" customHeight="1"/>
-    <x:row r="491" ht="15" customHeight="1"/>
-    <x:row r="492" ht="15" customHeight="1"/>
-    <x:row r="493" ht="15" customHeight="1"/>
-    <x:row r="494" ht="15" customHeight="1"/>
-    <x:row r="495" ht="15" customHeight="1"/>
-    <x:row r="496" ht="15" customHeight="1"/>
-    <x:row r="497" ht="15" customHeight="1"/>
-    <x:row r="498" ht="15" customHeight="1"/>
-    <x:row r="499" ht="15" customHeight="1"/>
-    <x:row r="500" ht="15" customHeight="1"/>
+    <x:row r="30">
+      <x:c r="A30" s="29"/>
+      <x:c r="B30" s="29"/>
+      <x:c r="C30" s="29"/>
+      <x:c r="D30" s="29"/>
+      <x:c r="E30" s="29"/>
+      <x:c r="F30" s="29"/>
+      <x:c r="G30" s="29"/>
+      <x:c r="H30" s="29"/>
+      <x:c r="I30" s="29"/>
+      <x:c r="J30" s="29"/>
+      <x:c r="K30" s="29"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:K500">
-    <x:cfRule type="expression" dxfId="11" priority="1">
-      <x:formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=0)</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="12" priority="2">
-      <x:formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=1)</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R312756fb74b54147"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5b1a72fb6a848d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update MICCAI DS Springer LNCS 16489 in publication masters
</commit_message>
<xml_diff>
--- a/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
+++ b/profile_private/Mineo_Raffaele_PublicationsMetadata.xlsx
@@ -2220,12 +2220,12 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>International Conference on Medical Image Computing and Computer-Assisted Intervention</t>
+          <t xml:space="preserve">Medical Image Computing and Computer Assisted Intervention -- MICCAI 2025 Doctoral Symposium; Lecture Notes in Computer Science, vol. 16489 (Springer)</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>MICCAI</t>
+          <t xml:space="preserve">MICCAI DS</t>
         </is>
       </c>
       <c r="E28" s="28" t="inlineStr">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="F28" s="28" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="G28" s="30" t="inlineStr">
         <is>
@@ -2243,11 +2243,13 @@
       </c>
       <c r="H28" s="30" t="inlineStr">
         <is>
-          <t>@inproceedings{mineo2025advancing,
+          <t xml:space="preserve">@inproceedings{mineo2027advancing,
   title={Advancing Healthcare with Multimodal AI: Enhanced Diagnosis, Cognitive Monitoring, and Inclusive Medical Communication},
   author={Mineo, Raffaele},
-  booktitle={International Conference on Medical Image Computing and Computer-Assisted Intervention},
-  year={2026},
+  booktitle={Medical Image Computing and Computer Assisted Intervention -- MICCAI 2025 Doctoral Symposium},
+  series={Lecture Notes in Computer Science},
+  volume={16489},
+  year={2027},
   organization={Springer}
 }</t>
         </is>

</xml_diff>